<commit_message>
Add SHADOW (DGE) and SHADOW_MIMIC from World Bank Informal Economy Database
- Downloaded official WB Informal Economy Database (Elgin et al. 2021)
- Filled SHADOW/SHADOW_MIMIC for Kazakhstan, Kyrgyz Republic, Tajikistan (2004-2020)
- Uzbekistan & Turkmenistan absent from DGE/MIMIC sheets -> left blank, flagged in READ_ME
- Coverage ends 2020; 2021-2022 blank
- merge_shadow.py documents the extraction
</commit_message>
<xml_diff>
--- a/DFS_data_FILLED.xlsx
+++ b/DFS_data_FILLED.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +35,10 @@
     <font>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -91,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -100,6 +104,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -465,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -478,9 +483,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -537,9 +539,6 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -565,6 +564,48 @@
       <c r="A15" t="inlineStr">
         <is>
           <t>A blank cell = missing data. It was left empty on purpose; no numbers were fabricated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>UPDATE - SHADOW now filled from World Bank Informal Economy Database (Elgin et al. 2021):</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - DGE (SHADOW) and MIMIC (SHADOW_MIMIC) filled for Kazakhstan, Kyrgyz Republic, Tajikistan, 2004-2020.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Database coverage ends in 2020, so 2021-2022 are blank (genuinely unavailable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - CRITICAL: Uzbekistan and Turkmenistan are NOT in the DGE/MIMIC sheets of this database.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Their SHADOW is blank. Source them from Medina &amp; Schneider (2018, IMF WP 18/17) appendix, or another series.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - This means the paper's main dependent variable is missing for 2 of the 5 core countries - a real feasibility issue to resolve.</t>
         </is>
       </c>
     </row>
@@ -733,8 +774,12 @@
       <c r="B2" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
+      <c r="C2" s="5" t="n">
+        <v>38.7009</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>41.3817</v>
+      </c>
       <c r="E2" s="5" t="n">
         <v>13.9087</v>
       </c>
@@ -790,8 +835,12 @@
       <c r="B3" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
+      <c r="C3" s="5" t="n">
+        <v>38.7384</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>40.9105</v>
+      </c>
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
@@ -845,8 +894,12 @@
       <c r="B4" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
+      <c r="C4" s="5" t="n">
+        <v>38.6245</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>40.0984</v>
+      </c>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
@@ -900,8 +953,12 @@
       <c r="B5" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
+      <c r="C5" s="5" t="n">
+        <v>38.4002</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>40.0649</v>
+      </c>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
@@ -955,8 +1012,12 @@
       <c r="B6" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
+      <c r="C6" s="5" t="n">
+        <v>38.2936</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>39.5908</v>
+      </c>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
@@ -1010,8 +1071,12 @@
       <c r="B7" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="4" t="n"/>
+      <c r="C7" s="5" t="n">
+        <v>37.9138</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>40.1043</v>
+      </c>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
@@ -1065,8 +1130,12 @@
       <c r="B8" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
+      <c r="C8" s="5" t="n">
+        <v>37.8459</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>39.4754</v>
+      </c>
       <c r="E8" s="5" t="n">
         <v>15.7124</v>
       </c>
@@ -1122,8 +1191,12 @@
       <c r="B9" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
+      <c r="C9" s="5" t="n">
+        <v>37.7151</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>39.0293</v>
+      </c>
       <c r="E9" s="5" t="n">
         <v>18.2578</v>
       </c>
@@ -1181,8 +1254,12 @@
       <c r="B10" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
+      <c r="C10" s="5" t="n">
+        <v>37.5983</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>39.2145</v>
+      </c>
       <c r="E10" s="5" t="n">
         <v>13.3121</v>
       </c>
@@ -1238,8 +1315,12 @@
       <c r="B11" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
+      <c r="C11" s="5" t="n">
+        <v>37.5761</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>38.543</v>
+      </c>
       <c r="E11" s="5" t="n">
         <v>16.0302</v>
       </c>
@@ -1295,8 +1376,12 @@
       <c r="B12" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
+      <c r="C12" s="5" t="n">
+        <v>36.896</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>38.295</v>
+      </c>
       <c r="E12" s="5" t="n">
         <v>14.1934</v>
       </c>
@@ -1356,8 +1441,12 @@
       <c r="B13" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
+      <c r="C13" s="5" t="n">
+        <v>36.9701</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>38.6224</v>
+      </c>
       <c r="E13" s="5" t="n">
         <v>9.835699999999999</v>
       </c>
@@ -1413,8 +1502,12 @@
       <c r="B14" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
+      <c r="C14" s="5" t="n">
+        <v>36.6046</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>38.6415</v>
+      </c>
       <c r="E14" s="5" t="n">
         <v>9.924300000000001</v>
       </c>
@@ -1470,8 +1563,12 @@
       <c r="B15" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
+      <c r="C15" s="5" t="n">
+        <v>36.0469</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>38.0948</v>
+      </c>
       <c r="E15" s="5" t="n">
         <v>10.303</v>
       </c>
@@ -1531,8 +1628,12 @@
       <c r="B16" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
+      <c r="C16" s="5" t="n">
+        <v>36.1346</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>37.1794</v>
+      </c>
       <c r="E16" s="5" t="n">
         <v>11.7178</v>
       </c>
@@ -1588,8 +1689,12 @@
       <c r="B17" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
+      <c r="C17" s="5" t="n">
+        <v>35.7794</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>37.2346</v>
+      </c>
       <c r="E17" s="5" t="n">
         <v>11.7869</v>
       </c>
@@ -1645,8 +1750,12 @@
       <c r="B18" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
+      <c r="C18" s="5" t="n">
+        <v>35.4727</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>38.3889</v>
+      </c>
       <c r="E18" s="5" t="n">
         <v>8.3188</v>
       </c>
@@ -1820,8 +1929,12 @@
       <c r="B21" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
+      <c r="C21" s="5" t="n">
+        <v>38.8296</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>40.0354</v>
+      </c>
       <c r="E21" s="5" t="n"/>
       <c r="F21" s="5" t="n"/>
       <c r="G21" s="5" t="n"/>
@@ -1875,8 +1988,12 @@
       <c r="B22" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
+      <c r="C22" s="5" t="n">
+        <v>39.1466</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>39.7818</v>
+      </c>
       <c r="E22" s="5" t="n"/>
       <c r="F22" s="5" t="n"/>
       <c r="G22" s="5" t="n"/>
@@ -1930,8 +2047,12 @@
       <c r="B23" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
+      <c r="C23" s="5" t="n">
+        <v>38.933</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>39.9025</v>
+      </c>
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n"/>
       <c r="G23" s="5" t="n"/>
@@ -1985,8 +2106,12 @@
       <c r="B24" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="4" t="n"/>
+      <c r="C24" s="5" t="n">
+        <v>38.8009</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>39.0296</v>
+      </c>
       <c r="E24" s="5" t="n"/>
       <c r="F24" s="5" t="n"/>
       <c r="G24" s="5" t="n"/>
@@ -2040,8 +2165,12 @@
       <c r="B25" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
+      <c r="C25" s="5" t="n">
+        <v>38.5255</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>38.7334</v>
+      </c>
       <c r="E25" s="5" t="n"/>
       <c r="F25" s="5" t="n"/>
       <c r="G25" s="5" t="n"/>
@@ -2095,8 +2224,12 @@
       <c r="B26" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
+      <c r="C26" s="5" t="n">
+        <v>38.0458</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>39.1544</v>
+      </c>
       <c r="E26" s="5" t="n"/>
       <c r="F26" s="5" t="n"/>
       <c r="G26" s="5" t="n"/>
@@ -2150,8 +2283,12 @@
       <c r="B27" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
+      <c r="C27" s="5" t="n">
+        <v>37.5493</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>39.0695</v>
+      </c>
       <c r="E27" s="5" t="n"/>
       <c r="F27" s="5" t="n"/>
       <c r="G27" s="5" t="n"/>
@@ -2205,8 +2342,12 @@
       <c r="B28" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
+      <c r="C28" s="5" t="n">
+        <v>37.1553</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>38.7456</v>
+      </c>
       <c r="E28" s="5" t="n"/>
       <c r="F28" s="5" t="n">
         <v>3.7573</v>
@@ -2262,8 +2403,12 @@
       <c r="B29" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
+      <c r="C29" s="5" t="n">
+        <v>36.7708</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>39.6338</v>
+      </c>
       <c r="E29" s="5" t="n"/>
       <c r="F29" s="5" t="n"/>
       <c r="G29" s="5" t="n"/>
@@ -2317,8 +2462,12 @@
       <c r="B30" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
+      <c r="C30" s="5" t="n">
+        <v>36.7102</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>38.2765</v>
+      </c>
       <c r="E30" s="5" t="n"/>
       <c r="F30" s="5" t="n"/>
       <c r="G30" s="5" t="n"/>
@@ -2372,8 +2521,12 @@
       <c r="B31" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
+      <c r="C31" s="5" t="n">
+        <v>36.3669</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>37.7415</v>
+      </c>
       <c r="E31" s="5" t="n">
         <v>17.5487</v>
       </c>
@@ -2433,8 +2586,12 @@
       <c r="B32" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
+      <c r="C32" s="5" t="n">
+        <v>35.8534</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>37.5703</v>
+      </c>
       <c r="E32" s="5" t="n">
         <v>16.8017</v>
       </c>
@@ -2490,8 +2647,12 @@
       <c r="B33" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="4" t="n"/>
+      <c r="C33" s="5" t="n">
+        <v>35.4168</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>37.1226</v>
+      </c>
       <c r="E33" s="5" t="n">
         <v>16.9492</v>
       </c>
@@ -2547,8 +2708,12 @@
       <c r="B34" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
+      <c r="C34" s="5" t="n">
+        <v>34.5402</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>36.5701</v>
+      </c>
       <c r="E34" s="5" t="n">
         <v>17.0463</v>
       </c>
@@ -2608,8 +2773,12 @@
       <c r="B35" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
+      <c r="C35" s="5" t="n">
+        <v>34.2123</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>36.3599</v>
+      </c>
       <c r="E35" s="5" t="n">
         <v>17.9989</v>
       </c>
@@ -2665,8 +2834,12 @@
       <c r="B36" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="4" t="n"/>
+      <c r="C36" s="5" t="n">
+        <v>33.7516</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>36.0072</v>
+      </c>
       <c r="E36" s="5" t="n">
         <v>15.9638</v>
       </c>
@@ -2722,8 +2895,12 @@
       <c r="B37" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
+      <c r="C37" s="5" t="n">
+        <v>33.185</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>37.6041</v>
+      </c>
       <c r="E37" s="5" t="n">
         <v>14.0363</v>
       </c>
@@ -2897,8 +3074,12 @@
       <c r="B40" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
+      <c r="C40" s="5" t="n">
+        <v>40.0794</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>42.206</v>
+      </c>
       <c r="E40" s="5" t="n">
         <v>9.821</v>
       </c>
@@ -2950,8 +3131,12 @@
       <c r="B41" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="4" t="n"/>
+      <c r="C41" s="5" t="n">
+        <v>40.4902</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>42.2759</v>
+      </c>
       <c r="E41" s="5" t="n"/>
       <c r="F41" s="5" t="n"/>
       <c r="G41" s="5" t="n"/>
@@ -3003,8 +3188,12 @@
       <c r="B42" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C42" s="4" t="n"/>
-      <c r="D42" s="4" t="n"/>
+      <c r="C42" s="5" t="n">
+        <v>40.778</v>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>41.7016</v>
+      </c>
       <c r="E42" s="5" t="n"/>
       <c r="F42" s="5" t="n"/>
       <c r="G42" s="5" t="n"/>
@@ -3056,8 +3245,12 @@
       <c r="B43" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C43" s="4" t="n"/>
-      <c r="D43" s="4" t="n"/>
+      <c r="C43" s="5" t="n">
+        <v>41.0031</v>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>41.2537</v>
+      </c>
       <c r="E43" s="5" t="n"/>
       <c r="F43" s="5" t="n"/>
       <c r="G43" s="5" t="n"/>
@@ -3111,8 +3304,12 @@
       <c r="B44" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
+      <c r="C44" s="5" t="n">
+        <v>41.1581</v>
+      </c>
+      <c r="D44" s="5" t="n">
+        <v>40.857</v>
+      </c>
       <c r="E44" s="5" t="n"/>
       <c r="F44" s="5" t="n"/>
       <c r="G44" s="5" t="n"/>
@@ -3166,8 +3363,12 @@
       <c r="B45" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C45" s="4" t="n"/>
-      <c r="D45" s="4" t="n"/>
+      <c r="C45" s="5" t="n">
+        <v>41.3139</v>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>41.1989</v>
+      </c>
       <c r="E45" s="5" t="n"/>
       <c r="F45" s="5" t="n"/>
       <c r="G45" s="5" t="n"/>
@@ -3221,8 +3422,12 @@
       <c r="B46" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C46" s="4" t="n"/>
-      <c r="D46" s="4" t="n"/>
+      <c r="C46" s="5" t="n">
+        <v>41.539</v>
+      </c>
+      <c r="D46" s="5" t="n">
+        <v>40.8445</v>
+      </c>
       <c r="E46" s="5" t="n"/>
       <c r="F46" s="5" t="n"/>
       <c r="G46" s="5" t="n"/>
@@ -3276,8 +3481,12 @@
       <c r="B47" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="4" t="n"/>
+      <c r="C47" s="5" t="n">
+        <v>41.475</v>
+      </c>
+      <c r="D47" s="5" t="n">
+        <v>40.7656</v>
+      </c>
       <c r="E47" s="5" t="n"/>
       <c r="F47" s="5" t="n">
         <v>2.5349</v>
@@ -3333,8 +3542,12 @@
       <c r="B48" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C48" s="4" t="n"/>
-      <c r="D48" s="4" t="n"/>
+      <c r="C48" s="5" t="n">
+        <v>42.0564</v>
+      </c>
+      <c r="D48" s="5" t="n">
+        <v>40.295</v>
+      </c>
       <c r="E48" s="5" t="n"/>
       <c r="F48" s="5" t="n"/>
       <c r="G48" s="5" t="n"/>
@@ -3388,8 +3601,12 @@
       <c r="B49" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C49" s="4" t="n"/>
-      <c r="D49" s="4" t="n"/>
+      <c r="C49" s="5" t="n">
+        <v>42.4303</v>
+      </c>
+      <c r="D49" s="5" t="n">
+        <v>40.2008</v>
+      </c>
       <c r="E49" s="5" t="n"/>
       <c r="F49" s="5" t="n"/>
       <c r="G49" s="5" t="n"/>
@@ -3443,8 +3660,12 @@
       <c r="B50" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C50" s="4" t="n"/>
-      <c r="D50" s="4" t="n"/>
+      <c r="C50" s="5" t="n">
+        <v>42.2822</v>
+      </c>
+      <c r="D50" s="5" t="n">
+        <v>39.7462</v>
+      </c>
       <c r="E50" s="5" t="n"/>
       <c r="F50" s="5" t="n">
         <v>11.4592</v>
@@ -3502,8 +3723,12 @@
       <c r="B51" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="4" t="n"/>
+      <c r="C51" s="5" t="n">
+        <v>43.011</v>
+      </c>
+      <c r="D51" s="5" t="n">
+        <v>39.4062</v>
+      </c>
       <c r="E51" s="5" t="n"/>
       <c r="F51" s="5" t="n"/>
       <c r="G51" s="5" t="n"/>
@@ -3557,8 +3782,12 @@
       <c r="B52" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="4" t="n"/>
+      <c r="C52" s="5" t="n">
+        <v>43.2744</v>
+      </c>
+      <c r="D52" s="5" t="n">
+        <v>38.8824</v>
+      </c>
       <c r="E52" s="5" t="n"/>
       <c r="F52" s="5" t="n"/>
       <c r="G52" s="5" t="n"/>
@@ -3612,8 +3841,12 @@
       <c r="B53" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="4" t="n"/>
+      <c r="C53" s="5" t="n">
+        <v>43.0029</v>
+      </c>
+      <c r="D53" s="5" t="n">
+        <v>38.6427</v>
+      </c>
       <c r="E53" s="5" t="n"/>
       <c r="F53" s="5" t="n">
         <v>47.0244</v>
@@ -3669,8 +3902,12 @@
       <c r="B54" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C54" s="4" t="n"/>
-      <c r="D54" s="4" t="n"/>
+      <c r="C54" s="5" t="n">
+        <v>42.9983</v>
+      </c>
+      <c r="D54" s="5" t="n">
+        <v>38.485</v>
+      </c>
       <c r="E54" s="5" t="n"/>
       <c r="F54" s="5" t="n"/>
       <c r="G54" s="5" t="n"/>
@@ -3720,8 +3957,12 @@
       <c r="B55" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
+      <c r="C55" s="5" t="n">
+        <v>43.2154</v>
+      </c>
+      <c r="D55" s="5" t="n">
+        <v>37.5825</v>
+      </c>
       <c r="E55" s="5" t="n"/>
       <c r="F55" s="5" t="n"/>
       <c r="G55" s="5" t="n"/>
@@ -3773,8 +4014,12 @@
       <c r="B56" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C56" s="4" t="n"/>
-      <c r="D56" s="4" t="n"/>
+      <c r="C56" s="5" t="n">
+        <v>43.002</v>
+      </c>
+      <c r="D56" s="5" t="n">
+        <v>37.6737</v>
+      </c>
       <c r="E56" s="5" t="n"/>
       <c r="F56" s="5" t="n"/>
       <c r="G56" s="5" t="n"/>
@@ -6068,8 +6313,12 @@
       <c r="B2" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
+      <c r="C2" s="5" t="n">
+        <v>34.0685</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>34.926</v>
+      </c>
       <c r="E2" s="5" t="n">
         <v>17.4267</v>
       </c>
@@ -6123,8 +6372,12 @@
       <c r="B3" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
+      <c r="C3" s="5" t="n">
+        <v>33.7752</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>34.7569</v>
+      </c>
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
@@ -6178,8 +6431,12 @@
       <c r="B4" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
+      <c r="C4" s="5" t="n">
+        <v>33.3872</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>34.3284</v>
+      </c>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
@@ -6231,8 +6488,12 @@
       <c r="B5" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
+      <c r="C5" s="5" t="n">
+        <v>32.9001</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>34.2056</v>
+      </c>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
@@ -6286,8 +6547,12 @@
       <c r="B6" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
+      <c r="C6" s="5" t="n">
+        <v>32.1643</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>33.7954</v>
+      </c>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
@@ -6341,8 +6606,12 @@
       <c r="B7" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="4" t="n"/>
+      <c r="C7" s="5" t="n">
+        <v>31.2854</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>33.9664</v>
+      </c>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
@@ -6396,8 +6665,12 @@
       <c r="B8" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
+      <c r="C8" s="5" t="n">
+        <v>30.8495</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>33.8801</v>
+      </c>
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
@@ -6451,8 +6724,12 @@
       <c r="B9" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
+      <c r="C9" s="5" t="n">
+        <v>30.6074</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>33.6508</v>
+      </c>
       <c r="E9" s="5" t="n">
         <v>17.9067</v>
       </c>
@@ -6510,8 +6787,12 @@
       <c r="B10" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
+      <c r="C10" s="5" t="n">
+        <v>30.5458</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>33.546</v>
+      </c>
       <c r="E10" s="5" t="n">
         <v>17.5879</v>
       </c>
@@ -6567,8 +6848,12 @@
       <c r="B11" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
+      <c r="C11" s="5" t="n">
+        <v>29.9724</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>33.8653</v>
+      </c>
       <c r="E11" s="5" t="n">
         <v>16.4765</v>
       </c>
@@ -6624,8 +6909,12 @@
       <c r="B12" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
+      <c r="C12" s="5" t="n">
+        <v>29.7679</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>33.8607</v>
+      </c>
       <c r="E12" s="5" t="n">
         <v>18.2081</v>
       </c>
@@ -6685,8 +6974,12 @@
       <c r="B13" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
+      <c r="C13" s="5" t="n">
+        <v>29.8274</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>33.7438</v>
+      </c>
       <c r="E13" s="5" t="n">
         <v>18.3813</v>
       </c>
@@ -6742,8 +7035,12 @@
       <c r="B14" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
+      <c r="C14" s="5" t="n">
+        <v>29.9466</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>33.3905</v>
+      </c>
       <c r="E14" s="5" t="n">
         <v>17.4032</v>
       </c>
@@ -6799,8 +7096,12 @@
       <c r="B15" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
+      <c r="C15" s="5" t="n">
+        <v>29.9669</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>33.0118</v>
+      </c>
       <c r="E15" s="5" t="n">
         <v>18.5477</v>
       </c>
@@ -6860,8 +7161,12 @@
       <c r="B16" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
+      <c r="C16" s="5" t="n">
+        <v>29.9187</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>32.5539</v>
+      </c>
       <c r="E16" s="5" t="n">
         <v>18.277</v>
       </c>
@@ -6917,8 +7222,12 @@
       <c r="B17" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
+      <c r="C17" s="5" t="n">
+        <v>29.7245</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>32.4233</v>
+      </c>
       <c r="E17" s="5" t="n">
         <v>17.931</v>
       </c>
@@ -6974,8 +7283,12 @@
       <c r="B18" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
+      <c r="C18" s="5" t="n">
+        <v>29.3367</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>32.8291</v>
+      </c>
       <c r="E18" s="5" t="n">
         <v>16.8955</v>
       </c>
@@ -7149,8 +7462,12 @@
       <c r="B21" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
+      <c r="C21" s="5" t="n">
+        <v>44.2381</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>45.7934</v>
+      </c>
       <c r="E21" s="5" t="n">
         <v>13.9964</v>
       </c>
@@ -7206,8 +7523,12 @@
       <c r="B22" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
+      <c r="C22" s="5" t="n">
+        <v>43.5052</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>45.0198</v>
+      </c>
       <c r="E22" s="5" t="n">
         <v>14.3357</v>
       </c>
@@ -7263,8 +7584,12 @@
       <c r="B23" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
+      <c r="C23" s="5" t="n">
+        <v>42.2737</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>44.6173</v>
+      </c>
       <c r="E23" s="5" t="n">
         <v>14.396</v>
       </c>
@@ -7318,8 +7643,12 @@
       <c r="B24" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="4" t="n"/>
+      <c r="C24" s="5" t="n">
+        <v>41.1006</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>44.1505</v>
+      </c>
       <c r="E24" s="5" t="n">
         <v>15.9625</v>
       </c>
@@ -7375,8 +7704,12 @@
       <c r="B25" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
+      <c r="C25" s="5" t="n">
+        <v>39.9882</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>42.7413</v>
+      </c>
       <c r="E25" s="5" t="n">
         <v>17.3218</v>
       </c>
@@ -7432,8 +7765,12 @@
       <c r="B26" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
+      <c r="C26" s="5" t="n">
+        <v>38.9532</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>44.0077</v>
+      </c>
       <c r="E26" s="5" t="n">
         <v>16.5059</v>
       </c>
@@ -7489,8 +7826,12 @@
       <c r="B27" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
+      <c r="C27" s="5" t="n">
+        <v>38.3545</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>43.9872</v>
+      </c>
       <c r="E27" s="5" t="n">
         <v>17.0701</v>
       </c>
@@ -7546,8 +7887,12 @@
       <c r="B28" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
+      <c r="C28" s="5" t="n">
+        <v>37.7506</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>43.6819</v>
+      </c>
       <c r="E28" s="5" t="n">
         <v>17.2194</v>
       </c>
@@ -7605,8 +7950,12 @@
       <c r="B29" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
+      <c r="C29" s="5" t="n">
+        <v>37.5061</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>43.2033</v>
+      </c>
       <c r="E29" s="5" t="n">
         <v>17.4916</v>
       </c>
@@ -7662,8 +8011,12 @@
       <c r="B30" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
+      <c r="C30" s="5" t="n">
+        <v>37.2692</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>43.1251</v>
+      </c>
       <c r="E30" s="5" t="n">
         <v>21.5862</v>
       </c>
@@ -7719,8 +8072,12 @@
       <c r="B31" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
+      <c r="C31" s="5" t="n">
+        <v>36.5299</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>43.2678</v>
+      </c>
       <c r="E31" s="5" t="n">
         <v>21.5992</v>
       </c>
@@ -7780,8 +8137,12 @@
       <c r="B32" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
+      <c r="C32" s="5" t="n">
+        <v>36.2212</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>43.3836</v>
+      </c>
       <c r="E32" s="5" t="n">
         <v>20.9312</v>
       </c>
@@ -7837,8 +8198,12 @@
       <c r="B33" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="4" t="n"/>
+      <c r="C33" s="5" t="n">
+        <v>35.6658</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>43.4115</v>
+      </c>
       <c r="E33" s="5" t="n">
         <v>21.2774</v>
       </c>
@@ -7894,8 +8259,12 @@
       <c r="B34" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
+      <c r="C34" s="5" t="n">
+        <v>35.3125</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>42.7821</v>
+      </c>
       <c r="E34" s="5" t="n">
         <v>20.7807</v>
       </c>
@@ -7955,8 +8324,12 @@
       <c r="B35" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
+      <c r="C35" s="5" t="n">
+        <v>34.5871</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>42.3893</v>
+      </c>
       <c r="E35" s="5" t="n">
         <v>20.8701</v>
       </c>
@@ -8012,8 +8385,12 @@
       <c r="B36" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="4" t="n"/>
+      <c r="C36" s="5" t="n">
+        <v>34.6181</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>42.195</v>
+      </c>
       <c r="E36" s="5" t="n">
         <v>22.2852</v>
       </c>
@@ -8069,8 +8446,12 @@
       <c r="B37" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
+      <c r="C37" s="5" t="n">
+        <v>33.9738</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>43.5617</v>
+      </c>
       <c r="E37" s="5" t="n">
         <v>21.8604</v>
       </c>
@@ -8244,8 +8625,12 @@
       <c r="B40" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
+      <c r="C40" s="5" t="n">
+        <v>54.4475</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>58.3953</v>
+      </c>
       <c r="E40" s="5" t="n"/>
       <c r="F40" s="5" t="n"/>
       <c r="G40" s="5" t="n"/>
@@ -8295,8 +8680,12 @@
       <c r="B41" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="4" t="n"/>
+      <c r="C41" s="5" t="n">
+        <v>54.0077</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>57.2318</v>
+      </c>
       <c r="E41" s="5" t="n"/>
       <c r="F41" s="5" t="n"/>
       <c r="G41" s="5" t="n"/>
@@ -8348,8 +8737,12 @@
       <c r="B42" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C42" s="4" t="n"/>
-      <c r="D42" s="4" t="n"/>
+      <c r="C42" s="5" t="n">
+        <v>52.9784</v>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>55.7652</v>
+      </c>
       <c r="E42" s="5" t="n"/>
       <c r="F42" s="5" t="n"/>
       <c r="G42" s="5" t="n"/>
@@ -8403,8 +8796,12 @@
       <c r="B43" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C43" s="4" t="n"/>
-      <c r="D43" s="4" t="n"/>
+      <c r="C43" s="5" t="n">
+        <v>52.0001</v>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>54.942</v>
+      </c>
       <c r="E43" s="5" t="n"/>
       <c r="F43" s="5" t="n"/>
       <c r="G43" s="5" t="n"/>
@@ -8458,8 +8855,12 @@
       <c r="B44" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
+      <c r="C44" s="5" t="n">
+        <v>50.6912</v>
+      </c>
+      <c r="D44" s="5" t="n">
+        <v>54.2579</v>
+      </c>
       <c r="E44" s="5" t="n">
         <v>16.4212</v>
       </c>
@@ -8515,8 +8916,12 @@
       <c r="B45" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C45" s="4" t="n"/>
-      <c r="D45" s="4" t="n"/>
+      <c r="C45" s="5" t="n">
+        <v>49.6373</v>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>54.1194</v>
+      </c>
       <c r="E45" s="5" t="n">
         <v>14.1067</v>
       </c>
@@ -8572,8 +8977,12 @@
       <c r="B46" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C46" s="4" t="n"/>
-      <c r="D46" s="4" t="n"/>
+      <c r="C46" s="5" t="n">
+        <v>48.5824</v>
+      </c>
+      <c r="D46" s="5" t="n">
+        <v>53.925</v>
+      </c>
       <c r="E46" s="5" t="n">
         <v>12.1578</v>
       </c>
@@ -8629,8 +9038,12 @@
       <c r="B47" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="4" t="n"/>
+      <c r="C47" s="5" t="n">
+        <v>47.0616</v>
+      </c>
+      <c r="D47" s="5" t="n">
+        <v>53.914</v>
+      </c>
       <c r="E47" s="5" t="n">
         <v>12.2248</v>
       </c>
@@ -8688,8 +9101,12 @@
       <c r="B48" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C48" s="4" t="n"/>
-      <c r="D48" s="4" t="n"/>
+      <c r="C48" s="5" t="n">
+        <v>45.8224</v>
+      </c>
+      <c r="D48" s="5" t="n">
+        <v>53.8678</v>
+      </c>
       <c r="E48" s="5" t="n">
         <v>12.7786</v>
       </c>
@@ -8745,8 +9162,12 @@
       <c r="B49" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C49" s="4" t="n"/>
-      <c r="D49" s="4" t="n"/>
+      <c r="C49" s="5" t="n">
+        <v>44.5833</v>
+      </c>
+      <c r="D49" s="5" t="n">
+        <v>53.3785</v>
+      </c>
       <c r="E49" s="5" t="n">
         <v>13.3883</v>
       </c>
@@ -8802,8 +9223,12 @@
       <c r="B50" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C50" s="4" t="n"/>
-      <c r="D50" s="4" t="n"/>
+      <c r="C50" s="5" t="n">
+        <v>43.0566</v>
+      </c>
+      <c r="D50" s="5" t="n">
+        <v>53.3749</v>
+      </c>
       <c r="E50" s="5" t="n">
         <v>14.2125</v>
       </c>
@@ -8863,8 +9288,12 @@
       <c r="B51" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="4" t="n"/>
+      <c r="C51" s="5" t="n">
+        <v>42.1758</v>
+      </c>
+      <c r="D51" s="5" t="n">
+        <v>53.5522</v>
+      </c>
       <c r="E51" s="5" t="n">
         <v>15.6032</v>
       </c>
@@ -8920,8 +9349,12 @@
       <c r="B52" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="4" t="n"/>
+      <c r="C52" s="5" t="n">
+        <v>41.5273</v>
+      </c>
+      <c r="D52" s="5" t="n">
+        <v>53.8302</v>
+      </c>
       <c r="E52" s="5" t="n">
         <v>14.5203</v>
       </c>
@@ -8977,8 +9410,12 @@
       <c r="B53" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="4" t="n"/>
+      <c r="C53" s="5" t="n">
+        <v>40.7811</v>
+      </c>
+      <c r="D53" s="5" t="n">
+        <v>53.6832</v>
+      </c>
       <c r="E53" s="5" t="n">
         <v>13.1335</v>
       </c>
@@ -9038,8 +9475,12 @@
       <c r="B54" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C54" s="4" t="n"/>
-      <c r="D54" s="4" t="n"/>
+      <c r="C54" s="5" t="n">
+        <v>40.4981</v>
+      </c>
+      <c r="D54" s="5" t="n">
+        <v>53.4947</v>
+      </c>
       <c r="E54" s="5" t="n">
         <v>12.9436</v>
       </c>
@@ -9095,8 +9536,12 @@
       <c r="B55" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
+      <c r="C55" s="5" t="n">
+        <v>39.9669</v>
+      </c>
+      <c r="D55" s="5" t="n">
+        <v>53.4228</v>
+      </c>
       <c r="E55" s="5" t="n">
         <v>14.19</v>
       </c>
@@ -9152,8 +9597,12 @@
       <c r="B56" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C56" s="4" t="n"/>
-      <c r="D56" s="4" t="n"/>
+      <c r="C56" s="5" t="n">
+        <v>39.0533</v>
+      </c>
+      <c r="D56" s="5" t="n">
+        <v>54.8374</v>
+      </c>
       <c r="E56" s="5" t="n">
         <v>15.1856</v>
       </c>
@@ -9327,8 +9776,12 @@
       <c r="B59" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C59" s="4" t="n"/>
-      <c r="D59" s="4" t="n"/>
+      <c r="C59" s="5" t="n">
+        <v>44.1108</v>
+      </c>
+      <c r="D59" s="5" t="n">
+        <v>47.5956</v>
+      </c>
       <c r="E59" s="5" t="n">
         <v>18.3713</v>
       </c>
@@ -9384,8 +9837,12 @@
       <c r="B60" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C60" s="4" t="n"/>
-      <c r="D60" s="4" t="n"/>
+      <c r="C60" s="5" t="n">
+        <v>44.1014</v>
+      </c>
+      <c r="D60" s="5" t="n">
+        <v>47.2651</v>
+      </c>
       <c r="E60" s="5" t="n">
         <v>20.1497</v>
       </c>
@@ -9441,8 +9898,12 @@
       <c r="B61" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C61" s="4" t="n"/>
-      <c r="D61" s="4" t="n"/>
+      <c r="C61" s="5" t="n">
+        <v>43.7653</v>
+      </c>
+      <c r="D61" s="5" t="n">
+        <v>46.5608</v>
+      </c>
       <c r="E61" s="5" t="n">
         <v>22.2231</v>
       </c>
@@ -9498,8 +9959,12 @@
       <c r="B62" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C62" s="4" t="n"/>
-      <c r="D62" s="4" t="n"/>
+      <c r="C62" s="5" t="n">
+        <v>43.3004</v>
+      </c>
+      <c r="D62" s="5" t="n">
+        <v>46.0219</v>
+      </c>
       <c r="E62" s="5" t="n">
         <v>23.7267</v>
       </c>
@@ -9555,8 +10020,12 @@
       <c r="B63" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C63" s="4" t="n"/>
-      <c r="D63" s="4" t="n"/>
+      <c r="C63" s="5" t="n">
+        <v>42.8171</v>
+      </c>
+      <c r="D63" s="5" t="n">
+        <v>45.1255</v>
+      </c>
       <c r="E63" s="5" t="n">
         <v>25.3534</v>
       </c>
@@ -9612,8 +10081,12 @@
       <c r="B64" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C64" s="4" t="n"/>
-      <c r="D64" s="4" t="n"/>
+      <c r="C64" s="5" t="n">
+        <v>42.0455</v>
+      </c>
+      <c r="D64" s="5" t="n">
+        <v>45.1325</v>
+      </c>
       <c r="E64" s="5" t="n">
         <v>18.6295</v>
       </c>
@@ -9669,8 +10142,12 @@
       <c r="B65" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C65" s="4" t="n"/>
-      <c r="D65" s="4" t="n"/>
+      <c r="C65" s="5" t="n">
+        <v>41.2613</v>
+      </c>
+      <c r="D65" s="5" t="n">
+        <v>44.7181</v>
+      </c>
       <c r="E65" s="5" t="n">
         <v>16.3214</v>
       </c>
@@ -9726,8 +10203,12 @@
       <c r="B66" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C66" s="4" t="n"/>
-      <c r="D66" s="4" t="n"/>
+      <c r="C66" s="5" t="n">
+        <v>40.3898</v>
+      </c>
+      <c r="D66" s="5" t="n">
+        <v>43.8568</v>
+      </c>
       <c r="E66" s="5" t="n">
         <v>14.5091</v>
       </c>
@@ -9785,8 +10266,12 @@
       <c r="B67" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C67" s="4" t="n"/>
-      <c r="D67" s="4" t="n"/>
+      <c r="C67" s="5" t="n">
+        <v>39.7847</v>
+      </c>
+      <c r="D67" s="5" t="n">
+        <v>43.6753</v>
+      </c>
       <c r="E67" s="5" t="n">
         <v>14.663</v>
       </c>
@@ -9842,8 +10327,12 @@
       <c r="B68" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C68" s="4" t="n"/>
-      <c r="D68" s="4" t="n"/>
+      <c r="C68" s="5" t="n">
+        <v>39.4058</v>
+      </c>
+      <c r="D68" s="5" t="n">
+        <v>43.6049</v>
+      </c>
       <c r="E68" s="5" t="n">
         <v>13.355</v>
       </c>
@@ -9899,8 +10388,12 @@
       <c r="B69" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C69" s="4" t="n"/>
-      <c r="D69" s="4" t="n"/>
+      <c r="C69" s="5" t="n">
+        <v>38.5553</v>
+      </c>
+      <c r="D69" s="5" t="n">
+        <v>43.4018</v>
+      </c>
       <c r="E69" s="5" t="n">
         <v>12.6977</v>
       </c>
@@ -9960,8 +10453,12 @@
       <c r="B70" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C70" s="4" t="n"/>
-      <c r="D70" s="4" t="n"/>
+      <c r="C70" s="5" t="n">
+        <v>38.5641</v>
+      </c>
+      <c r="D70" s="5" t="n">
+        <v>42.9811</v>
+      </c>
       <c r="E70" s="5" t="n">
         <v>14.1731</v>
       </c>
@@ -10017,8 +10514,12 @@
       <c r="B71" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C71" s="4" t="n"/>
-      <c r="D71" s="4" t="n"/>
+      <c r="C71" s="5" t="n">
+        <v>38.229</v>
+      </c>
+      <c r="D71" s="5" t="n">
+        <v>43.2793</v>
+      </c>
       <c r="E71" s="5" t="n">
         <v>13.7882</v>
       </c>
@@ -10074,8 +10575,12 @@
       <c r="B72" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C72" s="4" t="n"/>
-      <c r="D72" s="4" t="n"/>
+      <c r="C72" s="5" t="n">
+        <v>37.6375</v>
+      </c>
+      <c r="D72" s="5" t="n">
+        <v>43.0476</v>
+      </c>
       <c r="E72" s="5" t="n">
         <v>13.019</v>
       </c>
@@ -10135,8 +10640,12 @@
       <c r="B73" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C73" s="4" t="n"/>
-      <c r="D73" s="4" t="n"/>
+      <c r="C73" s="5" t="n">
+        <v>37.5188</v>
+      </c>
+      <c r="D73" s="5" t="n">
+        <v>42.6945</v>
+      </c>
       <c r="E73" s="5" t="n">
         <v>14.6726</v>
       </c>
@@ -10192,8 +10701,12 @@
       <c r="B74" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C74" s="4" t="n"/>
-      <c r="D74" s="4" t="n"/>
+      <c r="C74" s="5" t="n">
+        <v>37.3029</v>
+      </c>
+      <c r="D74" s="5" t="n">
+        <v>42.5392</v>
+      </c>
       <c r="E74" s="5" t="n">
         <v>13.3015</v>
       </c>
@@ -10249,8 +10762,12 @@
       <c r="B75" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C75" s="4" t="n"/>
-      <c r="D75" s="4" t="n"/>
+      <c r="C75" s="5" t="n">
+        <v>36.7677</v>
+      </c>
+      <c r="D75" s="5" t="n">
+        <v>43.1005</v>
+      </c>
       <c r="E75" s="5" t="n">
         <v>12.0229</v>
       </c>
@@ -10420,8 +10937,12 @@
       <c r="B78" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C78" s="4" t="n"/>
-      <c r="D78" s="4" t="n"/>
+      <c r="C78" s="5" t="n">
+        <v>34.7983</v>
+      </c>
+      <c r="D78" s="5" t="n">
+        <v>34.0908</v>
+      </c>
       <c r="E78" s="5" t="n"/>
       <c r="F78" s="5" t="n"/>
       <c r="G78" s="5" t="n"/>
@@ -10471,8 +10992,12 @@
       <c r="B79" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C79" s="4" t="n"/>
-      <c r="D79" s="4" t="n"/>
+      <c r="C79" s="5" t="n">
+        <v>33.8796</v>
+      </c>
+      <c r="D79" s="5" t="n">
+        <v>33.5705</v>
+      </c>
       <c r="E79" s="5" t="n">
         <v>19.8861</v>
       </c>
@@ -10524,8 +11049,12 @@
       <c r="B80" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C80" s="4" t="n"/>
-      <c r="D80" s="4" t="n"/>
+      <c r="C80" s="5" t="n">
+        <v>33.2544</v>
+      </c>
+      <c r="D80" s="5" t="n">
+        <v>33.7206</v>
+      </c>
       <c r="E80" s="5" t="n">
         <v>21.69</v>
       </c>
@@ -10581,8 +11110,12 @@
       <c r="B81" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C81" s="4" t="n"/>
-      <c r="D81" s="4" t="n"/>
+      <c r="C81" s="5" t="n">
+        <v>32.8006</v>
+      </c>
+      <c r="D81" s="5" t="n">
+        <v>33.4629</v>
+      </c>
       <c r="E81" s="5" t="n">
         <v>21.3943</v>
       </c>
@@ -10638,8 +11171,12 @@
       <c r="B82" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C82" s="4" t="n"/>
-      <c r="D82" s="4" t="n"/>
+      <c r="C82" s="5" t="n">
+        <v>32.1341</v>
+      </c>
+      <c r="D82" s="5" t="n">
+        <v>32.8665</v>
+      </c>
       <c r="E82" s="5" t="n">
         <v>20.3021</v>
       </c>
@@ -10695,8 +11232,12 @@
       <c r="B83" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C83" s="4" t="n"/>
-      <c r="D83" s="4" t="n"/>
+      <c r="C83" s="5" t="n">
+        <v>31.6479</v>
+      </c>
+      <c r="D83" s="5" t="n">
+        <v>33.3289</v>
+      </c>
       <c r="E83" s="5" t="n">
         <v>18.9463</v>
       </c>
@@ -10752,8 +11293,12 @@
       <c r="B84" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C84" s="4" t="n"/>
-      <c r="D84" s="4" t="n"/>
+      <c r="C84" s="5" t="n">
+        <v>31.2542</v>
+      </c>
+      <c r="D84" s="5" t="n">
+        <v>33.4874</v>
+      </c>
       <c r="E84" s="5" t="n">
         <v>19.6857</v>
       </c>
@@ -10809,8 +11354,12 @@
       <c r="B85" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C85" s="4" t="n"/>
-      <c r="D85" s="4" t="n"/>
+      <c r="C85" s="5" t="n">
+        <v>30.7265</v>
+      </c>
+      <c r="D85" s="5" t="n">
+        <v>33.4375</v>
+      </c>
       <c r="E85" s="5" t="n">
         <v>20.3057</v>
       </c>
@@ -10868,8 +11417,12 @@
       <c r="B86" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C86" s="4" t="n"/>
-      <c r="D86" s="4" t="n"/>
+      <c r="C86" s="5" t="n">
+        <v>30.3049</v>
+      </c>
+      <c r="D86" s="5" t="n">
+        <v>33.4122</v>
+      </c>
       <c r="E86" s="5" t="n">
         <v>20.4775</v>
       </c>
@@ -10925,8 +11478,12 @@
       <c r="B87" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C87" s="4" t="n"/>
-      <c r="D87" s="4" t="n"/>
+      <c r="C87" s="5" t="n">
+        <v>29.9666</v>
+      </c>
+      <c r="D87" s="5" t="n">
+        <v>33.0644</v>
+      </c>
       <c r="E87" s="5" t="n">
         <v>19.7515</v>
       </c>
@@ -10982,8 +11539,12 @@
       <c r="B88" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C88" s="4" t="n"/>
-      <c r="D88" s="4" t="n"/>
+      <c r="C88" s="5" t="n">
+        <v>29.613</v>
+      </c>
+      <c r="D88" s="5" t="n">
+        <v>33.0111</v>
+      </c>
       <c r="E88" s="5" t="n">
         <v>19.7779</v>
       </c>
@@ -11043,8 +11604,12 @@
       <c r="B89" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C89" s="4" t="n"/>
-      <c r="D89" s="4" t="n"/>
+      <c r="C89" s="5" t="n">
+        <v>29.3739</v>
+      </c>
+      <c r="D89" s="5" t="n">
+        <v>32.6818</v>
+      </c>
       <c r="E89" s="5" t="n">
         <v>19.7</v>
       </c>
@@ -11100,8 +11665,12 @@
       <c r="B90" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C90" s="4" t="n"/>
-      <c r="D90" s="4" t="n"/>
+      <c r="C90" s="5" t="n">
+        <v>29.1626</v>
+      </c>
+      <c r="D90" s="5" t="n">
+        <v>31.9989</v>
+      </c>
       <c r="E90" s="5" t="n">
         <v>19.7137</v>
       </c>
@@ -11157,8 +11726,12 @@
       <c r="B91" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C91" s="4" t="n"/>
-      <c r="D91" s="4" t="n"/>
+      <c r="C91" s="5" t="n">
+        <v>29.2119</v>
+      </c>
+      <c r="D91" s="5" t="n">
+        <v>31.2462</v>
+      </c>
       <c r="E91" s="5" t="n">
         <v>19.9877</v>
       </c>
@@ -11218,8 +11791,12 @@
       <c r="B92" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C92" s="4" t="n"/>
-      <c r="D92" s="4" t="n"/>
+      <c r="C92" s="5" t="n">
+        <v>28.9843</v>
+      </c>
+      <c r="D92" s="5" t="n">
+        <v>30.7766</v>
+      </c>
       <c r="E92" s="5" t="n">
         <v>20.141</v>
       </c>
@@ -11275,8 +11852,12 @@
       <c r="B93" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C93" s="4" t="n"/>
-      <c r="D93" s="4" t="n"/>
+      <c r="C93" s="5" t="n">
+        <v>28.7681</v>
+      </c>
+      <c r="D93" s="5" t="n">
+        <v>30.3014</v>
+      </c>
       <c r="E93" s="5" t="n">
         <v>19.8266</v>
       </c>
@@ -11332,8 +11913,12 @@
       <c r="B94" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C94" s="4" t="n"/>
-      <c r="D94" s="4" t="n"/>
+      <c r="C94" s="5" t="n">
+        <v>28.4014</v>
+      </c>
+      <c r="D94" s="5" t="n">
+        <v>31.027</v>
+      </c>
       <c r="E94" s="5" t="n">
         <v>18.7506</v>
       </c>
@@ -11507,8 +12092,12 @@
       <c r="B97" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C97" s="4" t="n"/>
-      <c r="D97" s="4" t="n"/>
+      <c r="C97" s="5" t="n">
+        <v>34.8429</v>
+      </c>
+      <c r="D97" s="5" t="n">
+        <v>35.5479</v>
+      </c>
       <c r="E97" s="5" t="n">
         <v>21.0296</v>
       </c>
@@ -11564,8 +12153,12 @@
       <c r="B98" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C98" s="4" t="n"/>
-      <c r="D98" s="4" t="n"/>
+      <c r="C98" s="5" t="n">
+        <v>34.0866</v>
+      </c>
+      <c r="D98" s="5" t="n">
+        <v>34.8598</v>
+      </c>
       <c r="E98" s="5" t="n">
         <v>20.8855</v>
       </c>
@@ -11621,8 +12214,12 @@
       <c r="B99" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C99" s="4" t="n"/>
-      <c r="D99" s="4" t="n"/>
+      <c r="C99" s="5" t="n">
+        <v>33.3586</v>
+      </c>
+      <c r="D99" s="5" t="n">
+        <v>34.631</v>
+      </c>
       <c r="E99" s="5" t="n">
         <v>21.812</v>
       </c>
@@ -11678,8 +12275,12 @@
       <c r="B100" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C100" s="4" t="n"/>
-      <c r="D100" s="4" t="n"/>
+      <c r="C100" s="5" t="n">
+        <v>32.7005</v>
+      </c>
+      <c r="D100" s="5" t="n">
+        <v>33.8554</v>
+      </c>
       <c r="E100" s="5" t="n">
         <v>21.7606</v>
       </c>
@@ -11735,8 +12336,12 @@
       <c r="B101" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C101" s="4" t="n"/>
-      <c r="D101" s="4" t="n"/>
+      <c r="C101" s="5" t="n">
+        <v>31.6974</v>
+      </c>
+      <c r="D101" s="5" t="n">
+        <v>33.5619</v>
+      </c>
       <c r="E101" s="5" t="n">
         <v>21.9739</v>
       </c>
@@ -11792,8 +12397,12 @@
       <c r="B102" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C102" s="4" t="n"/>
-      <c r="D102" s="4" t="n"/>
+      <c r="C102" s="5" t="n">
+        <v>30.9083</v>
+      </c>
+      <c r="D102" s="5" t="n">
+        <v>33.5566</v>
+      </c>
       <c r="E102" s="5" t="n">
         <v>18.5865</v>
       </c>
@@ -11849,8 +12458,12 @@
       <c r="B103" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C103" s="4" t="n"/>
-      <c r="D103" s="4" t="n"/>
+      <c r="C103" s="5" t="n">
+        <v>30.1717</v>
+      </c>
+      <c r="D103" s="5" t="n">
+        <v>33.7961</v>
+      </c>
       <c r="E103" s="5" t="n">
         <v>17.8714</v>
       </c>
@@ -11906,8 +12519,12 @@
       <c r="B104" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C104" s="4" t="n"/>
-      <c r="D104" s="4" t="n"/>
+      <c r="C104" s="5" t="n">
+        <v>29.7026</v>
+      </c>
+      <c r="D104" s="5" t="n">
+        <v>33.5999</v>
+      </c>
       <c r="E104" s="5" t="n">
         <v>17.8827</v>
       </c>
@@ -11965,8 +12582,12 @@
       <c r="B105" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C105" s="4" t="n"/>
-      <c r="D105" s="4" t="n"/>
+      <c r="C105" s="5" t="n">
+        <v>29.3849</v>
+      </c>
+      <c r="D105" s="5" t="n">
+        <v>33.5908</v>
+      </c>
       <c r="E105" s="5" t="n">
         <v>18.3853</v>
       </c>
@@ -12022,8 +12643,12 @@
       <c r="B106" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C106" s="4" t="n"/>
-      <c r="D106" s="4" t="n"/>
+      <c r="C106" s="5" t="n">
+        <v>29.0233</v>
+      </c>
+      <c r="D106" s="5" t="n">
+        <v>33.8344</v>
+      </c>
       <c r="E106" s="5" t="n">
         <v>19.6863</v>
       </c>
@@ -12079,8 +12704,12 @@
       <c r="B107" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C107" s="4" t="n"/>
-      <c r="D107" s="4" t="n"/>
+      <c r="C107" s="5" t="n">
+        <v>28.8427</v>
+      </c>
+      <c r="D107" s="5" t="n">
+        <v>33.6153</v>
+      </c>
       <c r="E107" s="5" t="n">
         <v>19.5666</v>
       </c>
@@ -12140,8 +12769,12 @@
       <c r="B108" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C108" s="4" t="n"/>
-      <c r="D108" s="4" t="n"/>
+      <c r="C108" s="5" t="n">
+        <v>28.6872</v>
+      </c>
+      <c r="D108" s="5" t="n">
+        <v>32.9816</v>
+      </c>
       <c r="E108" s="5" t="n">
         <v>20.0778</v>
       </c>
@@ -12197,8 +12830,12 @@
       <c r="B109" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C109" s="4" t="n"/>
-      <c r="D109" s="4" t="n"/>
+      <c r="C109" s="5" t="n">
+        <v>28.4847</v>
+      </c>
+      <c r="D109" s="5" t="n">
+        <v>32.4583</v>
+      </c>
       <c r="E109" s="5" t="n">
         <v>20.333</v>
       </c>
@@ -12254,8 +12891,12 @@
       <c r="B110" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C110" s="4" t="n"/>
-      <c r="D110" s="4" t="n"/>
+      <c r="C110" s="5" t="n">
+        <v>28.4958</v>
+      </c>
+      <c r="D110" s="5" t="n">
+        <v>32.1244</v>
+      </c>
       <c r="E110" s="5" t="n">
         <v>20.5232</v>
       </c>
@@ -12315,8 +12956,12 @@
       <c r="B111" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C111" s="4" t="n"/>
-      <c r="D111" s="4" t="n"/>
+      <c r="C111" s="5" t="n">
+        <v>28.2373</v>
+      </c>
+      <c r="D111" s="5" t="n">
+        <v>31.9761</v>
+      </c>
       <c r="E111" s="5" t="n">
         <v>19.9835</v>
       </c>
@@ -12372,8 +13017,12 @@
       <c r="B112" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C112" s="4" t="n"/>
-      <c r="D112" s="4" t="n"/>
+      <c r="C112" s="5" t="n">
+        <v>28.1232</v>
+      </c>
+      <c r="D112" s="5" t="n">
+        <v>31.7999</v>
+      </c>
       <c r="E112" s="5" t="n">
         <v>20.5951</v>
       </c>
@@ -12429,8 +13078,12 @@
       <c r="B113" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C113" s="4" t="n"/>
-      <c r="D113" s="4" t="n"/>
+      <c r="C113" s="5" t="n">
+        <v>27.7557</v>
+      </c>
+      <c r="D113" s="5" t="n">
+        <v>32.7301</v>
+      </c>
       <c r="E113" s="5" t="n">
         <v>20.1967</v>
       </c>
@@ -12604,8 +13257,12 @@
       <c r="B116" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C116" s="4" t="n"/>
-      <c r="D116" s="4" t="n"/>
+      <c r="C116" s="5" t="n">
+        <v>30.9633</v>
+      </c>
+      <c r="D116" s="5" t="n">
+        <v>31.4864</v>
+      </c>
       <c r="E116" s="5" t="n">
         <v>20.8831</v>
       </c>
@@ -12659,8 +13316,12 @@
       <c r="B117" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C117" s="4" t="n"/>
-      <c r="D117" s="4" t="n"/>
+      <c r="C117" s="5" t="n">
+        <v>30.7478</v>
+      </c>
+      <c r="D117" s="5" t="n">
+        <v>31.1092</v>
+      </c>
       <c r="E117" s="5" t="n">
         <v>20.8852</v>
       </c>
@@ -12716,8 +13377,12 @@
       <c r="B118" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C118" s="4" t="n"/>
-      <c r="D118" s="4" t="n"/>
+      <c r="C118" s="5" t="n">
+        <v>30.6126</v>
+      </c>
+      <c r="D118" s="5" t="n">
+        <v>30.6046</v>
+      </c>
       <c r="E118" s="5" t="n">
         <v>21.456</v>
       </c>
@@ -12773,8 +13438,12 @@
       <c r="B119" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C119" s="4" t="n"/>
-      <c r="D119" s="4" t="n"/>
+      <c r="C119" s="5" t="n">
+        <v>30.4003</v>
+      </c>
+      <c r="D119" s="5" t="n">
+        <v>30.29</v>
+      </c>
       <c r="E119" s="5" t="n">
         <v>21.4886</v>
       </c>
@@ -12830,8 +13499,12 @@
       <c r="B120" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C120" s="4" t="n"/>
-      <c r="D120" s="4" t="n"/>
+      <c r="C120" s="5" t="n">
+        <v>30.1984</v>
+      </c>
+      <c r="D120" s="5" t="n">
+        <v>29.9359</v>
+      </c>
       <c r="E120" s="5" t="n">
         <v>21.2698</v>
       </c>
@@ -12887,8 +13560,12 @@
       <c r="B121" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C121" s="4" t="n"/>
-      <c r="D121" s="4" t="n"/>
+      <c r="C121" s="5" t="n">
+        <v>29.8793</v>
+      </c>
+      <c r="D121" s="5" t="n">
+        <v>30.8058</v>
+      </c>
       <c r="E121" s="5" t="n">
         <v>20.2772</v>
       </c>
@@ -12944,8 +13621,12 @@
       <c r="B122" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C122" s="4" t="n"/>
-      <c r="D122" s="4" t="n"/>
+      <c r="C122" s="5" t="n">
+        <v>29.5713</v>
+      </c>
+      <c r="D122" s="5" t="n">
+        <v>31.1202</v>
+      </c>
       <c r="E122" s="5" t="n">
         <v>20.281</v>
       </c>
@@ -13001,8 +13682,12 @@
       <c r="B123" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C123" s="4" t="n"/>
-      <c r="D123" s="4" t="n"/>
+      <c r="C123" s="5" t="n">
+        <v>29.2116</v>
+      </c>
+      <c r="D123" s="5" t="n">
+        <v>31.3159</v>
+      </c>
       <c r="E123" s="5" t="n">
         <v>19.6485</v>
       </c>
@@ -13060,8 +13745,12 @@
       <c r="B124" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C124" s="4" t="n"/>
-      <c r="D124" s="4" t="n"/>
+      <c r="C124" s="5" t="n">
+        <v>28.9821</v>
+      </c>
+      <c r="D124" s="5" t="n">
+        <v>31.5981</v>
+      </c>
       <c r="E124" s="5" t="n">
         <v>20.1296</v>
       </c>
@@ -13117,8 +13806,12 @@
       <c r="B125" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C125" s="4" t="n"/>
-      <c r="D125" s="4" t="n"/>
+      <c r="C125" s="5" t="n">
+        <v>28.7258</v>
+      </c>
+      <c r="D125" s="5" t="n">
+        <v>31.7134</v>
+      </c>
       <c r="E125" s="5" t="n">
         <v>20.5988</v>
       </c>
@@ -13174,8 +13867,12 @@
       <c r="B126" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C126" s="4" t="n"/>
-      <c r="D126" s="4" t="n"/>
+      <c r="C126" s="5" t="n">
+        <v>28.7723</v>
+      </c>
+      <c r="D126" s="5" t="n">
+        <v>31.7248</v>
+      </c>
       <c r="E126" s="5" t="n">
         <v>20.3827</v>
       </c>
@@ -13235,8 +13932,12 @@
       <c r="B127" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C127" s="4" t="n"/>
-      <c r="D127" s="4" t="n"/>
+      <c r="C127" s="5" t="n">
+        <v>28.8176</v>
+      </c>
+      <c r="D127" s="5" t="n">
+        <v>31.551</v>
+      </c>
       <c r="E127" s="5" t="n">
         <v>21.4161</v>
       </c>
@@ -13292,8 +13993,12 @@
       <c r="B128" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C128" s="4" t="n"/>
-      <c r="D128" s="4" t="n"/>
+      <c r="C128" s="5" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="D128" s="5" t="n">
+        <v>30.9101</v>
+      </c>
       <c r="E128" s="5" t="n">
         <v>21.9038</v>
       </c>
@@ -13349,8 +14054,12 @@
       <c r="B129" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C129" s="4" t="n"/>
-      <c r="D129" s="4" t="n"/>
+      <c r="C129" s="5" t="n">
+        <v>28.9008</v>
+      </c>
+      <c r="D129" s="5" t="n">
+        <v>30.3628</v>
+      </c>
       <c r="E129" s="5" t="n">
         <v>22.0182</v>
       </c>
@@ -13410,8 +14119,12 @@
       <c r="B130" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C130" s="4" t="n"/>
-      <c r="D130" s="4" t="n"/>
+      <c r="C130" s="5" t="n">
+        <v>28.871</v>
+      </c>
+      <c r="D130" s="5" t="n">
+        <v>29.8695</v>
+      </c>
       <c r="E130" s="5" t="n">
         <v>21.7868</v>
       </c>
@@ -13467,8 +14180,12 @@
       <c r="B131" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C131" s="4" t="n"/>
-      <c r="D131" s="4" t="n"/>
+      <c r="C131" s="5" t="n">
+        <v>28.8216</v>
+      </c>
+      <c r="D131" s="5" t="n">
+        <v>29.5044</v>
+      </c>
       <c r="E131" s="5" t="n">
         <v>21.9731</v>
       </c>
@@ -13524,8 +14241,12 @@
       <c r="B132" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C132" s="4" t="n"/>
-      <c r="D132" s="4" t="n"/>
+      <c r="C132" s="5" t="n">
+        <v>28.4241</v>
+      </c>
+      <c r="D132" s="5" t="n">
+        <v>30.6446</v>
+      </c>
       <c r="E132" s="5" t="n">
         <v>20.8752</v>
       </c>
@@ -13699,8 +14420,12 @@
       <c r="B135" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C135" s="4" t="n"/>
-      <c r="D135" s="4" t="n"/>
+      <c r="C135" s="5" t="n">
+        <v>64.84699999999999</v>
+      </c>
+      <c r="D135" s="5" t="n">
+        <v>67.3533</v>
+      </c>
       <c r="E135" s="5" t="n">
         <v>15.1023</v>
       </c>
@@ -13756,8 +14481,12 @@
       <c r="B136" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C136" s="4" t="n"/>
-      <c r="D136" s="4" t="n"/>
+      <c r="C136" s="5" t="n">
+        <v>63.9392</v>
+      </c>
+      <c r="D136" s="5" t="n">
+        <v>67.6174</v>
+      </c>
       <c r="E136" s="5" t="n">
         <v>16.5426</v>
       </c>
@@ -13813,8 +14542,12 @@
       <c r="B137" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C137" s="4" t="n"/>
-      <c r="D137" s="4" t="n"/>
+      <c r="C137" s="5" t="n">
+        <v>63.1918</v>
+      </c>
+      <c r="D137" s="5" t="n">
+        <v>66.8171</v>
+      </c>
       <c r="E137" s="5" t="n">
         <v>18.5701</v>
       </c>
@@ -13870,8 +14603,12 @@
       <c r="B138" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C138" s="4" t="n"/>
-      <c r="D138" s="4" t="n"/>
+      <c r="C138" s="5" t="n">
+        <v>62.1002</v>
+      </c>
+      <c r="D138" s="5" t="n">
+        <v>66.7804</v>
+      </c>
       <c r="E138" s="5" t="n">
         <v>20.9553</v>
       </c>
@@ -13927,8 +14664,12 @@
       <c r="B139" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C139" s="4" t="n"/>
-      <c r="D139" s="4" t="n"/>
+      <c r="C139" s="5" t="n">
+        <v>61.6726</v>
+      </c>
+      <c r="D139" s="5" t="n">
+        <v>67.8933</v>
+      </c>
       <c r="E139" s="5" t="n">
         <v>24.2245</v>
       </c>
@@ -13984,8 +14725,12 @@
       <c r="B140" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C140" s="4" t="n"/>
-      <c r="D140" s="4" t="n"/>
+      <c r="C140" s="5" t="n">
+        <v>61.859</v>
+      </c>
+      <c r="D140" s="5" t="n">
+        <v>67.98779999999999</v>
+      </c>
       <c r="E140" s="5" t="n">
         <v>23.5094</v>
       </c>
@@ -14041,8 +14786,12 @@
       <c r="B141" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C141" s="4" t="n"/>
-      <c r="D141" s="4" t="n"/>
+      <c r="C141" s="5" t="n">
+        <v>61.8207</v>
+      </c>
+      <c r="D141" s="5" t="n">
+        <v>67.02</v>
+      </c>
       <c r="E141" s="5" t="n">
         <v>21.1107</v>
       </c>
@@ -14098,8 +14847,12 @@
       <c r="B142" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C142" s="4" t="n"/>
-      <c r="D142" s="4" t="n"/>
+      <c r="C142" s="5" t="n">
+        <v>61.6233</v>
+      </c>
+      <c r="D142" s="5" t="n">
+        <v>65.8826</v>
+      </c>
       <c r="E142" s="5" t="n">
         <v>22.6614</v>
       </c>
@@ -14157,8 +14910,12 @@
       <c r="B143" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C143" s="4" t="n"/>
-      <c r="D143" s="4" t="n"/>
+      <c r="C143" s="5" t="n">
+        <v>61.4383</v>
+      </c>
+      <c r="D143" s="5" t="n">
+        <v>65.3599</v>
+      </c>
       <c r="E143" s="5" t="n">
         <v>23.0885</v>
       </c>
@@ -14214,8 +14971,12 @@
       <c r="B144" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C144" s="4" t="n"/>
-      <c r="D144" s="4" t="n"/>
+      <c r="C144" s="5" t="n">
+        <v>61.0834</v>
+      </c>
+      <c r="D144" s="5" t="n">
+        <v>65.05629999999999</v>
+      </c>
       <c r="E144" s="5" t="n">
         <v>22.0626</v>
       </c>
@@ -14271,8 +15032,12 @@
       <c r="B145" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C145" s="4" t="n"/>
-      <c r="D145" s="4" t="n"/>
+      <c r="C145" s="5" t="n">
+        <v>61.0478</v>
+      </c>
+      <c r="D145" s="5" t="n">
+        <v>64.4987</v>
+      </c>
       <c r="E145" s="5" t="n">
         <v>22.0531</v>
       </c>
@@ -14332,8 +15097,12 @@
       <c r="B146" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C146" s="4" t="n"/>
-      <c r="D146" s="4" t="n"/>
+      <c r="C146" s="5" t="n">
+        <v>60.8766</v>
+      </c>
+      <c r="D146" s="5" t="n">
+        <v>63.9471</v>
+      </c>
       <c r="E146" s="5" t="n">
         <v>22.3477</v>
       </c>
@@ -14389,8 +15158,12 @@
       <c r="B147" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C147" s="4" t="n"/>
-      <c r="D147" s="4" t="n"/>
+      <c r="C147" s="5" t="n">
+        <v>60.1282</v>
+      </c>
+      <c r="D147" s="5" t="n">
+        <v>63.8882</v>
+      </c>
       <c r="E147" s="5" t="n">
         <v>23.0424</v>
       </c>
@@ -14446,8 +15219,12 @@
       <c r="B148" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C148" s="4" t="n"/>
-      <c r="D148" s="4" t="n"/>
+      <c r="C148" s="5" t="n">
+        <v>59.8357</v>
+      </c>
+      <c r="D148" s="5" t="n">
+        <v>62.5503</v>
+      </c>
       <c r="E148" s="5" t="n">
         <v>23.0135</v>
       </c>
@@ -14507,8 +15284,12 @@
       <c r="B149" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C149" s="4" t="n"/>
-      <c r="D149" s="4" t="n"/>
+      <c r="C149" s="5" t="n">
+        <v>59.4199</v>
+      </c>
+      <c r="D149" s="5" t="n">
+        <v>61.6932</v>
+      </c>
       <c r="E149" s="5" t="n">
         <v>22.0479</v>
       </c>
@@ -14564,8 +15345,12 @@
       <c r="B150" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C150" s="4" t="n"/>
-      <c r="D150" s="4" t="n"/>
+      <c r="C150" s="5" t="n">
+        <v>58.7918</v>
+      </c>
+      <c r="D150" s="5" t="n">
+        <v>60.8236</v>
+      </c>
       <c r="E150" s="5" t="n">
         <v>22.8973</v>
       </c>
@@ -14621,8 +15406,12 @@
       <c r="B151" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C151" s="4" t="n"/>
-      <c r="D151" s="4" t="n"/>
+      <c r="C151" s="5" t="n">
+        <v>58.187</v>
+      </c>
+      <c r="D151" s="5" t="n">
+        <v>61.7879</v>
+      </c>
       <c r="E151" s="5" t="n">
         <v>21.1808</v>
       </c>
@@ -14796,8 +15585,12 @@
       <c r="B154" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C154" s="4" t="n"/>
-      <c r="D154" s="4" t="n"/>
+      <c r="C154" s="5" t="n">
+        <v>38.7009</v>
+      </c>
+      <c r="D154" s="5" t="n">
+        <v>41.3817</v>
+      </c>
       <c r="E154" s="5" t="n">
         <v>13.9087</v>
       </c>
@@ -14853,8 +15646,12 @@
       <c r="B155" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C155" s="4" t="n"/>
-      <c r="D155" s="4" t="n"/>
+      <c r="C155" s="5" t="n">
+        <v>38.7384</v>
+      </c>
+      <c r="D155" s="5" t="n">
+        <v>40.9105</v>
+      </c>
       <c r="E155" s="5" t="n"/>
       <c r="F155" s="5" t="n"/>
       <c r="G155" s="5" t="n"/>
@@ -14908,8 +15705,12 @@
       <c r="B156" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C156" s="4" t="n"/>
-      <c r="D156" s="4" t="n"/>
+      <c r="C156" s="5" t="n">
+        <v>38.6245</v>
+      </c>
+      <c r="D156" s="5" t="n">
+        <v>40.0984</v>
+      </c>
       <c r="E156" s="5" t="n"/>
       <c r="F156" s="5" t="n"/>
       <c r="G156" s="5" t="n"/>
@@ -14963,8 +15764,12 @@
       <c r="B157" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C157" s="4" t="n"/>
-      <c r="D157" s="4" t="n"/>
+      <c r="C157" s="5" t="n">
+        <v>38.4002</v>
+      </c>
+      <c r="D157" s="5" t="n">
+        <v>40.0649</v>
+      </c>
       <c r="E157" s="5" t="n"/>
       <c r="F157" s="5" t="n"/>
       <c r="G157" s="5" t="n"/>
@@ -15018,8 +15823,12 @@
       <c r="B158" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C158" s="4" t="n"/>
-      <c r="D158" s="4" t="n"/>
+      <c r="C158" s="5" t="n">
+        <v>38.2936</v>
+      </c>
+      <c r="D158" s="5" t="n">
+        <v>39.5908</v>
+      </c>
       <c r="E158" s="5" t="n"/>
       <c r="F158" s="5" t="n"/>
       <c r="G158" s="5" t="n"/>
@@ -15073,8 +15882,12 @@
       <c r="B159" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C159" s="4" t="n"/>
-      <c r="D159" s="4" t="n"/>
+      <c r="C159" s="5" t="n">
+        <v>37.9138</v>
+      </c>
+      <c r="D159" s="5" t="n">
+        <v>40.1043</v>
+      </c>
       <c r="E159" s="5" t="n"/>
       <c r="F159" s="5" t="n"/>
       <c r="G159" s="5" t="n"/>
@@ -15128,8 +15941,12 @@
       <c r="B160" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C160" s="4" t="n"/>
-      <c r="D160" s="4" t="n"/>
+      <c r="C160" s="5" t="n">
+        <v>37.8459</v>
+      </c>
+      <c r="D160" s="5" t="n">
+        <v>39.4754</v>
+      </c>
       <c r="E160" s="5" t="n">
         <v>15.7124</v>
       </c>
@@ -15185,8 +16002,12 @@
       <c r="B161" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C161" s="4" t="n"/>
-      <c r="D161" s="4" t="n"/>
+      <c r="C161" s="5" t="n">
+        <v>37.7151</v>
+      </c>
+      <c r="D161" s="5" t="n">
+        <v>39.0293</v>
+      </c>
       <c r="E161" s="5" t="n">
         <v>18.2578</v>
       </c>
@@ -15244,8 +16065,12 @@
       <c r="B162" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C162" s="4" t="n"/>
-      <c r="D162" s="4" t="n"/>
+      <c r="C162" s="5" t="n">
+        <v>37.5983</v>
+      </c>
+      <c r="D162" s="5" t="n">
+        <v>39.2145</v>
+      </c>
       <c r="E162" s="5" t="n">
         <v>13.3121</v>
       </c>
@@ -15301,8 +16126,12 @@
       <c r="B163" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C163" s="4" t="n"/>
-      <c r="D163" s="4" t="n"/>
+      <c r="C163" s="5" t="n">
+        <v>37.5761</v>
+      </c>
+      <c r="D163" s="5" t="n">
+        <v>38.543</v>
+      </c>
       <c r="E163" s="5" t="n">
         <v>16.0302</v>
       </c>
@@ -15358,8 +16187,12 @@
       <c r="B164" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C164" s="4" t="n"/>
-      <c r="D164" s="4" t="n"/>
+      <c r="C164" s="5" t="n">
+        <v>36.896</v>
+      </c>
+      <c r="D164" s="5" t="n">
+        <v>38.295</v>
+      </c>
       <c r="E164" s="5" t="n">
         <v>14.1934</v>
       </c>
@@ -15419,8 +16252,12 @@
       <c r="B165" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C165" s="4" t="n"/>
-      <c r="D165" s="4" t="n"/>
+      <c r="C165" s="5" t="n">
+        <v>36.9701</v>
+      </c>
+      <c r="D165" s="5" t="n">
+        <v>38.6224</v>
+      </c>
       <c r="E165" s="5" t="n">
         <v>9.835699999999999</v>
       </c>
@@ -15476,8 +16313,12 @@
       <c r="B166" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C166" s="4" t="n"/>
-      <c r="D166" s="4" t="n"/>
+      <c r="C166" s="5" t="n">
+        <v>36.6046</v>
+      </c>
+      <c r="D166" s="5" t="n">
+        <v>38.6415</v>
+      </c>
       <c r="E166" s="5" t="n">
         <v>9.924300000000001</v>
       </c>
@@ -15533,8 +16374,12 @@
       <c r="B167" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C167" s="4" t="n"/>
-      <c r="D167" s="4" t="n"/>
+      <c r="C167" s="5" t="n">
+        <v>36.0469</v>
+      </c>
+      <c r="D167" s="5" t="n">
+        <v>38.0948</v>
+      </c>
       <c r="E167" s="5" t="n">
         <v>10.303</v>
       </c>
@@ -15594,8 +16439,12 @@
       <c r="B168" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C168" s="4" t="n"/>
-      <c r="D168" s="4" t="n"/>
+      <c r="C168" s="5" t="n">
+        <v>36.1346</v>
+      </c>
+      <c r="D168" s="5" t="n">
+        <v>37.1794</v>
+      </c>
       <c r="E168" s="5" t="n">
         <v>11.7178</v>
       </c>
@@ -15651,8 +16500,12 @@
       <c r="B169" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C169" s="4" t="n"/>
-      <c r="D169" s="4" t="n"/>
+      <c r="C169" s="5" t="n">
+        <v>35.7794</v>
+      </c>
+      <c r="D169" s="5" t="n">
+        <v>37.2346</v>
+      </c>
       <c r="E169" s="5" t="n">
         <v>11.7869</v>
       </c>
@@ -15708,8 +16561,12 @@
       <c r="B170" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C170" s="4" t="n"/>
-      <c r="D170" s="4" t="n"/>
+      <c r="C170" s="5" t="n">
+        <v>35.4727</v>
+      </c>
+      <c r="D170" s="5" t="n">
+        <v>38.3889</v>
+      </c>
       <c r="E170" s="5" t="n">
         <v>8.3188</v>
       </c>
@@ -15883,8 +16740,12 @@
       <c r="B173" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C173" s="4" t="n"/>
-      <c r="D173" s="4" t="n"/>
+      <c r="C173" s="5" t="n">
+        <v>38.8296</v>
+      </c>
+      <c r="D173" s="5" t="n">
+        <v>40.0354</v>
+      </c>
       <c r="E173" s="5" t="n"/>
       <c r="F173" s="5" t="n"/>
       <c r="G173" s="5" t="n"/>
@@ -15938,8 +16799,12 @@
       <c r="B174" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C174" s="4" t="n"/>
-      <c r="D174" s="4" t="n"/>
+      <c r="C174" s="5" t="n">
+        <v>39.1466</v>
+      </c>
+      <c r="D174" s="5" t="n">
+        <v>39.7818</v>
+      </c>
       <c r="E174" s="5" t="n"/>
       <c r="F174" s="5" t="n"/>
       <c r="G174" s="5" t="n"/>
@@ -15993,8 +16858,12 @@
       <c r="B175" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C175" s="4" t="n"/>
-      <c r="D175" s="4" t="n"/>
+      <c r="C175" s="5" t="n">
+        <v>38.933</v>
+      </c>
+      <c r="D175" s="5" t="n">
+        <v>39.9025</v>
+      </c>
       <c r="E175" s="5" t="n"/>
       <c r="F175" s="5" t="n"/>
       <c r="G175" s="5" t="n"/>
@@ -16048,8 +16917,12 @@
       <c r="B176" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C176" s="4" t="n"/>
-      <c r="D176" s="4" t="n"/>
+      <c r="C176" s="5" t="n">
+        <v>38.8009</v>
+      </c>
+      <c r="D176" s="5" t="n">
+        <v>39.0296</v>
+      </c>
       <c r="E176" s="5" t="n"/>
       <c r="F176" s="5" t="n"/>
       <c r="G176" s="5" t="n"/>
@@ -16103,8 +16976,12 @@
       <c r="B177" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C177" s="4" t="n"/>
-      <c r="D177" s="4" t="n"/>
+      <c r="C177" s="5" t="n">
+        <v>38.5255</v>
+      </c>
+      <c r="D177" s="5" t="n">
+        <v>38.7334</v>
+      </c>
       <c r="E177" s="5" t="n"/>
       <c r="F177" s="5" t="n"/>
       <c r="G177" s="5" t="n"/>
@@ -16158,8 +17035,12 @@
       <c r="B178" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C178" s="4" t="n"/>
-      <c r="D178" s="4" t="n"/>
+      <c r="C178" s="5" t="n">
+        <v>38.0458</v>
+      </c>
+      <c r="D178" s="5" t="n">
+        <v>39.1544</v>
+      </c>
       <c r="E178" s="5" t="n"/>
       <c r="F178" s="5" t="n"/>
       <c r="G178" s="5" t="n"/>
@@ -16213,8 +17094,12 @@
       <c r="B179" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C179" s="4" t="n"/>
-      <c r="D179" s="4" t="n"/>
+      <c r="C179" s="5" t="n">
+        <v>37.5493</v>
+      </c>
+      <c r="D179" s="5" t="n">
+        <v>39.0695</v>
+      </c>
       <c r="E179" s="5" t="n"/>
       <c r="F179" s="5" t="n"/>
       <c r="G179" s="5" t="n"/>
@@ -16268,8 +17153,12 @@
       <c r="B180" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C180" s="4" t="n"/>
-      <c r="D180" s="4" t="n"/>
+      <c r="C180" s="5" t="n">
+        <v>37.1553</v>
+      </c>
+      <c r="D180" s="5" t="n">
+        <v>38.7456</v>
+      </c>
       <c r="E180" s="5" t="n"/>
       <c r="F180" s="5" t="n">
         <v>3.7573</v>
@@ -16325,8 +17214,12 @@
       <c r="B181" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C181" s="4" t="n"/>
-      <c r="D181" s="4" t="n"/>
+      <c r="C181" s="5" t="n">
+        <v>36.7708</v>
+      </c>
+      <c r="D181" s="5" t="n">
+        <v>39.6338</v>
+      </c>
       <c r="E181" s="5" t="n"/>
       <c r="F181" s="5" t="n"/>
       <c r="G181" s="5" t="n"/>
@@ -16380,8 +17273,12 @@
       <c r="B182" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C182" s="4" t="n"/>
-      <c r="D182" s="4" t="n"/>
+      <c r="C182" s="5" t="n">
+        <v>36.7102</v>
+      </c>
+      <c r="D182" s="5" t="n">
+        <v>38.2765</v>
+      </c>
       <c r="E182" s="5" t="n"/>
       <c r="F182" s="5" t="n"/>
       <c r="G182" s="5" t="n"/>
@@ -16435,8 +17332,12 @@
       <c r="B183" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C183" s="4" t="n"/>
-      <c r="D183" s="4" t="n"/>
+      <c r="C183" s="5" t="n">
+        <v>36.3669</v>
+      </c>
+      <c r="D183" s="5" t="n">
+        <v>37.7415</v>
+      </c>
       <c r="E183" s="5" t="n">
         <v>17.5487</v>
       </c>
@@ -16496,8 +17397,12 @@
       <c r="B184" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C184" s="4" t="n"/>
-      <c r="D184" s="4" t="n"/>
+      <c r="C184" s="5" t="n">
+        <v>35.8534</v>
+      </c>
+      <c r="D184" s="5" t="n">
+        <v>37.5703</v>
+      </c>
       <c r="E184" s="5" t="n">
         <v>16.8017</v>
       </c>
@@ -16553,8 +17458,12 @@
       <c r="B185" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C185" s="4" t="n"/>
-      <c r="D185" s="4" t="n"/>
+      <c r="C185" s="5" t="n">
+        <v>35.4168</v>
+      </c>
+      <c r="D185" s="5" t="n">
+        <v>37.1226</v>
+      </c>
       <c r="E185" s="5" t="n">
         <v>16.9492</v>
       </c>
@@ -16610,8 +17519,12 @@
       <c r="B186" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C186" s="4" t="n"/>
-      <c r="D186" s="4" t="n"/>
+      <c r="C186" s="5" t="n">
+        <v>34.5402</v>
+      </c>
+      <c r="D186" s="5" t="n">
+        <v>36.5701</v>
+      </c>
       <c r="E186" s="5" t="n">
         <v>17.0463</v>
       </c>
@@ -16671,8 +17584,12 @@
       <c r="B187" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C187" s="4" t="n"/>
-      <c r="D187" s="4" t="n"/>
+      <c r="C187" s="5" t="n">
+        <v>34.2123</v>
+      </c>
+      <c r="D187" s="5" t="n">
+        <v>36.3599</v>
+      </c>
       <c r="E187" s="5" t="n">
         <v>17.9989</v>
       </c>
@@ -16728,8 +17645,12 @@
       <c r="B188" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C188" s="4" t="n"/>
-      <c r="D188" s="4" t="n"/>
+      <c r="C188" s="5" t="n">
+        <v>33.7516</v>
+      </c>
+      <c r="D188" s="5" t="n">
+        <v>36.0072</v>
+      </c>
       <c r="E188" s="5" t="n">
         <v>15.9638</v>
       </c>
@@ -16785,8 +17706,12 @@
       <c r="B189" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C189" s="4" t="n"/>
-      <c r="D189" s="4" t="n"/>
+      <c r="C189" s="5" t="n">
+        <v>33.185</v>
+      </c>
+      <c r="D189" s="5" t="n">
+        <v>37.6041</v>
+      </c>
       <c r="E189" s="5" t="n">
         <v>14.0363</v>
       </c>
@@ -16960,8 +17885,12 @@
       <c r="B192" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C192" s="4" t="n"/>
-      <c r="D192" s="4" t="n"/>
+      <c r="C192" s="5" t="n">
+        <v>44.4275</v>
+      </c>
+      <c r="D192" s="5" t="n">
+        <v>44.2407</v>
+      </c>
       <c r="E192" s="5" t="n">
         <v>16.3574</v>
       </c>
@@ -17017,8 +17946,12 @@
       <c r="B193" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C193" s="4" t="n"/>
-      <c r="D193" s="4" t="n"/>
+      <c r="C193" s="5" t="n">
+        <v>44.6533</v>
+      </c>
+      <c r="D193" s="5" t="n">
+        <v>43.8157</v>
+      </c>
       <c r="E193" s="5" t="n">
         <v>18.4853</v>
       </c>
@@ -17074,8 +18007,12 @@
       <c r="B194" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C194" s="4" t="n"/>
-      <c r="D194" s="4" t="n"/>
+      <c r="C194" s="5" t="n">
+        <v>44.3007</v>
+      </c>
+      <c r="D194" s="5" t="n">
+        <v>44.075</v>
+      </c>
       <c r="E194" s="5" t="n">
         <v>19.5712</v>
       </c>
@@ -17131,8 +18068,12 @@
       <c r="B195" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C195" s="4" t="n"/>
-      <c r="D195" s="4" t="n"/>
+      <c r="C195" s="5" t="n">
+        <v>44.099</v>
+      </c>
+      <c r="D195" s="5" t="n">
+        <v>43.333</v>
+      </c>
       <c r="E195" s="5" t="n">
         <v>20.5665</v>
       </c>
@@ -17188,8 +18129,12 @@
       <c r="B196" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C196" s="4" t="n"/>
-      <c r="D196" s="4" t="n"/>
+      <c r="C196" s="5" t="n">
+        <v>43.9571</v>
+      </c>
+      <c r="D196" s="5" t="n">
+        <v>42.6788</v>
+      </c>
       <c r="E196" s="5" t="n">
         <v>20.4459</v>
       </c>
@@ -17245,8 +18190,12 @@
       <c r="B197" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C197" s="4" t="n"/>
-      <c r="D197" s="4" t="n"/>
+      <c r="C197" s="5" t="n">
+        <v>43.5322</v>
+      </c>
+      <c r="D197" s="5" t="n">
+        <v>43.893</v>
+      </c>
       <c r="E197" s="5" t="n">
         <v>17.6853</v>
       </c>
@@ -17302,8 +18251,12 @@
       <c r="B198" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C198" s="4" t="n"/>
-      <c r="D198" s="4" t="n"/>
+      <c r="C198" s="5" t="n">
+        <v>43.2136</v>
+      </c>
+      <c r="D198" s="5" t="n">
+        <v>43.6694</v>
+      </c>
       <c r="E198" s="5" t="n">
         <v>15.1606</v>
       </c>
@@ -17359,8 +18312,12 @@
       <c r="B199" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C199" s="4" t="n"/>
-      <c r="D199" s="4" t="n"/>
+      <c r="C199" s="5" t="n">
+        <v>43.1295</v>
+      </c>
+      <c r="D199" s="5" t="n">
+        <v>42.8951</v>
+      </c>
       <c r="E199" s="5" t="n">
         <v>15.2403</v>
       </c>
@@ -17418,8 +18375,12 @@
       <c r="B200" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C200" s="4" t="n"/>
-      <c r="D200" s="4" t="n"/>
+      <c r="C200" s="5" t="n">
+        <v>43.0626</v>
+      </c>
+      <c r="D200" s="5" t="n">
+        <v>42.6245</v>
+      </c>
       <c r="E200" s="5" t="n">
         <v>15.5953</v>
       </c>
@@ -17475,8 +18436,12 @@
       <c r="B201" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C201" s="4" t="n"/>
-      <c r="D201" s="4" t="n"/>
+      <c r="C201" s="5" t="n">
+        <v>43.5676</v>
+      </c>
+      <c r="D201" s="5" t="n">
+        <v>41.6728</v>
+      </c>
       <c r="E201" s="5" t="n">
         <v>15.4696</v>
       </c>
@@ -17532,8 +18497,12 @@
       <c r="B202" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C202" s="4" t="n"/>
-      <c r="D202" s="4" t="n"/>
+      <c r="C202" s="5" t="n">
+        <v>43.2456</v>
+      </c>
+      <c r="D202" s="5" t="n">
+        <v>40.7818</v>
+      </c>
       <c r="E202" s="5" t="n">
         <v>16.8288</v>
       </c>
@@ -17593,8 +18562,12 @@
       <c r="B203" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C203" s="4" t="n"/>
-      <c r="D203" s="4" t="n"/>
+      <c r="C203" s="5" t="n">
+        <v>43.9689</v>
+      </c>
+      <c r="D203" s="5" t="n">
+        <v>41.3559</v>
+      </c>
       <c r="E203" s="5" t="n">
         <v>16.291</v>
       </c>
@@ -17650,8 +18623,12 @@
       <c r="B204" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C204" s="4" t="n"/>
-      <c r="D204" s="4" t="n"/>
+      <c r="C204" s="5" t="n">
+        <v>44.0635</v>
+      </c>
+      <c r="D204" s="5" t="n">
+        <v>41.1624</v>
+      </c>
       <c r="E204" s="5" t="n">
         <v>16.4301</v>
       </c>
@@ -17707,8 +18684,12 @@
       <c r="B205" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C205" s="4" t="n"/>
-      <c r="D205" s="4" t="n"/>
+      <c r="C205" s="5" t="n">
+        <v>43.5457</v>
+      </c>
+      <c r="D205" s="5" t="n">
+        <v>40.6545</v>
+      </c>
       <c r="E205" s="5" t="n">
         <v>17.7274</v>
       </c>
@@ -17768,8 +18749,12 @@
       <c r="B206" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C206" s="4" t="n"/>
-      <c r="D206" s="4" t="n"/>
+      <c r="C206" s="5" t="n">
+        <v>43.8613</v>
+      </c>
+      <c r="D206" s="5" t="n">
+        <v>40.1996</v>
+      </c>
       <c r="E206" s="5" t="n">
         <v>18.0141</v>
       </c>
@@ -17825,8 +18810,12 @@
       <c r="B207" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C207" s="4" t="n"/>
-      <c r="D207" s="4" t="n"/>
+      <c r="C207" s="5" t="n">
+        <v>43.6291</v>
+      </c>
+      <c r="D207" s="5" t="n">
+        <v>39.7785</v>
+      </c>
       <c r="E207" s="5" t="n">
         <v>17.6563</v>
       </c>
@@ -17882,8 +18871,12 @@
       <c r="B208" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C208" s="4" t="n"/>
-      <c r="D208" s="4" t="n"/>
+      <c r="C208" s="5" t="n">
+        <v>42.7831</v>
+      </c>
+      <c r="D208" s="5" t="n">
+        <v>40.4242</v>
+      </c>
       <c r="E208" s="5" t="n">
         <v>17.9099</v>
       </c>
@@ -19088,8 +20081,12 @@
       <c r="B230" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C230" s="4" t="n"/>
-      <c r="D230" s="4" t="n"/>
+      <c r="C230" s="5" t="n">
+        <v>34.4877</v>
+      </c>
+      <c r="D230" s="5" t="n">
+        <v>38.2384</v>
+      </c>
       <c r="E230" s="5" t="n"/>
       <c r="F230" s="5" t="n"/>
       <c r="G230" s="5" t="n"/>
@@ -19139,8 +20136,12 @@
       <c r="B231" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C231" s="4" t="n"/>
-      <c r="D231" s="4" t="n"/>
+      <c r="C231" s="5" t="n">
+        <v>34.836</v>
+      </c>
+      <c r="D231" s="5" t="n">
+        <v>37.7806</v>
+      </c>
       <c r="E231" s="5" t="n">
         <v>18.4251</v>
       </c>
@@ -19196,8 +20197,12 @@
       <c r="B232" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C232" s="4" t="n"/>
-      <c r="D232" s="4" t="n"/>
+      <c r="C232" s="5" t="n">
+        <v>34.9388</v>
+      </c>
+      <c r="D232" s="5" t="n">
+        <v>37.4133</v>
+      </c>
       <c r="E232" s="5" t="n">
         <v>18.0827</v>
       </c>
@@ -19253,8 +20258,12 @@
       <c r="B233" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C233" s="4" t="n"/>
-      <c r="D233" s="4" t="n"/>
+      <c r="C233" s="5" t="n">
+        <v>34.9003</v>
+      </c>
+      <c r="D233" s="5" t="n">
+        <v>37.049</v>
+      </c>
       <c r="E233" s="5" t="n">
         <v>19.0748</v>
       </c>
@@ -19310,8 +20319,12 @@
       <c r="B234" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C234" s="4" t="n"/>
-      <c r="D234" s="4" t="n"/>
+      <c r="C234" s="5" t="n">
+        <v>34.987</v>
+      </c>
+      <c r="D234" s="5" t="n">
+        <v>36.9505</v>
+      </c>
       <c r="E234" s="5" t="n">
         <v>18.5239</v>
       </c>
@@ -19367,8 +20380,12 @@
       <c r="B235" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C235" s="4" t="n"/>
-      <c r="D235" s="4" t="n"/>
+      <c r="C235" s="5" t="n">
+        <v>35.0413</v>
+      </c>
+      <c r="D235" s="5" t="n">
+        <v>36.9896</v>
+      </c>
       <c r="E235" s="5" t="n">
         <v>17.1296</v>
       </c>
@@ -19424,8 +20441,12 @@
       <c r="B236" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C236" s="4" t="n"/>
-      <c r="D236" s="4" t="n"/>
+      <c r="C236" s="5" t="n">
+        <v>34.639</v>
+      </c>
+      <c r="D236" s="5" t="n">
+        <v>36.602</v>
+      </c>
       <c r="E236" s="5" t="n">
         <v>16.8657</v>
       </c>
@@ -19481,8 +20502,12 @@
       <c r="B237" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C237" s="4" t="n"/>
-      <c r="D237" s="4" t="n"/>
+      <c r="C237" s="5" t="n">
+        <v>34.3292</v>
+      </c>
+      <c r="D237" s="5" t="n">
+        <v>36.3755</v>
+      </c>
       <c r="E237" s="5" t="n">
         <v>16.9997</v>
       </c>
@@ -19540,8 +20565,12 @@
       <c r="B238" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C238" s="4" t="n"/>
-      <c r="D238" s="4" t="n"/>
+      <c r="C238" s="5" t="n">
+        <v>34.1046</v>
+      </c>
+      <c r="D238" s="5" t="n">
+        <v>36.4882</v>
+      </c>
       <c r="E238" s="5" t="n">
         <v>16.4167</v>
       </c>
@@ -19597,8 +20626,12 @@
       <c r="B239" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C239" s="4" t="n"/>
-      <c r="D239" s="4" t="n"/>
+      <c r="C239" s="5" t="n">
+        <v>34.2068</v>
+      </c>
+      <c r="D239" s="5" t="n">
+        <v>35.9102</v>
+      </c>
       <c r="E239" s="5" t="n">
         <v>15.669</v>
       </c>
@@ -19654,8 +20687,12 @@
       <c r="B240" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C240" s="4" t="n"/>
-      <c r="D240" s="4" t="n"/>
+      <c r="C240" s="5" t="n">
+        <v>34.0794</v>
+      </c>
+      <c r="D240" s="5" t="n">
+        <v>35.4423</v>
+      </c>
       <c r="E240" s="5" t="n">
         <v>16.2353</v>
       </c>
@@ -19715,8 +20752,12 @@
       <c r="B241" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C241" s="4" t="n"/>
-      <c r="D241" s="4" t="n"/>
+      <c r="C241" s="5" t="n">
+        <v>33.8359</v>
+      </c>
+      <c r="D241" s="5" t="n">
+        <v>35.0156</v>
+      </c>
       <c r="E241" s="5" t="n">
         <v>16.8182</v>
       </c>
@@ -19772,8 +20813,12 @@
       <c r="B242" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C242" s="4" t="n"/>
-      <c r="D242" s="4" t="n"/>
+      <c r="C242" s="5" t="n">
+        <v>33.679</v>
+      </c>
+      <c r="D242" s="5" t="n">
+        <v>34.3228</v>
+      </c>
       <c r="E242" s="5" t="n">
         <v>16.9512</v>
       </c>
@@ -19829,8 +20874,12 @@
       <c r="B243" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C243" s="4" t="n"/>
-      <c r="D243" s="4" t="n"/>
+      <c r="C243" s="5" t="n">
+        <v>33.4255</v>
+      </c>
+      <c r="D243" s="5" t="n">
+        <v>34.0333</v>
+      </c>
       <c r="E243" s="5" t="n">
         <v>17.1611</v>
       </c>
@@ -19890,8 +20939,12 @@
       <c r="B244" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C244" s="4" t="n"/>
-      <c r="D244" s="4" t="n"/>
+      <c r="C244" s="5" t="n">
+        <v>33.1964</v>
+      </c>
+      <c r="D244" s="5" t="n">
+        <v>33.6447</v>
+      </c>
       <c r="E244" s="5" t="n">
         <v>17.5749</v>
       </c>
@@ -19947,8 +21000,12 @@
       <c r="B245" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C245" s="4" t="n"/>
-      <c r="D245" s="4" t="n"/>
+      <c r="C245" s="5" t="n">
+        <v>33.1354</v>
+      </c>
+      <c r="D245" s="5" t="n">
+        <v>33.2678</v>
+      </c>
       <c r="E245" s="5" t="n">
         <v>17.0833</v>
       </c>
@@ -20004,8 +21061,12 @@
       <c r="B246" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C246" s="4" t="n"/>
-      <c r="D246" s="4" t="n"/>
+      <c r="C246" s="5" t="n">
+        <v>32.6939</v>
+      </c>
+      <c r="D246" s="5" t="n">
+        <v>34.0679</v>
+      </c>
       <c r="E246" s="5" t="n">
         <v>16.127</v>
       </c>
@@ -20179,8 +21240,12 @@
       <c r="B249" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C249" s="4" t="n"/>
-      <c r="D249" s="4" t="n"/>
+      <c r="C249" s="5" t="n">
+        <v>31.5096</v>
+      </c>
+      <c r="D249" s="5" t="n">
+        <v>33.5775</v>
+      </c>
       <c r="E249" s="5" t="n">
         <v>17.4213</v>
       </c>
@@ -20236,8 +21301,12 @@
       <c r="B250" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C250" s="4" t="n"/>
-      <c r="D250" s="4" t="n"/>
+      <c r="C250" s="5" t="n">
+        <v>31.1743</v>
+      </c>
+      <c r="D250" s="5" t="n">
+        <v>33.361</v>
+      </c>
       <c r="E250" s="5" t="n">
         <v>17.4681</v>
       </c>
@@ -20293,8 +21362,12 @@
       <c r="B251" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C251" s="4" t="n"/>
-      <c r="D251" s="4" t="n"/>
+      <c r="C251" s="5" t="n">
+        <v>30.9024</v>
+      </c>
+      <c r="D251" s="5" t="n">
+        <v>33.0077</v>
+      </c>
       <c r="E251" s="5" t="n">
         <v>17.9471</v>
       </c>
@@ -20350,8 +21423,12 @@
       <c r="B252" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C252" s="4" t="n"/>
-      <c r="D252" s="4" t="n"/>
+      <c r="C252" s="5" t="n">
+        <v>30.2002</v>
+      </c>
+      <c r="D252" s="5" t="n">
+        <v>32.3963</v>
+      </c>
       <c r="E252" s="5" t="n">
         <v>17.5395</v>
       </c>
@@ -20407,8 +21484,12 @@
       <c r="B253" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C253" s="4" t="n"/>
-      <c r="D253" s="4" t="n"/>
+      <c r="C253" s="5" t="n">
+        <v>29.3711</v>
+      </c>
+      <c r="D253" s="5" t="n">
+        <v>31.8867</v>
+      </c>
       <c r="E253" s="5" t="n">
         <v>16.7861</v>
       </c>
@@ -20464,8 +21545,12 @@
       <c r="B254" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C254" s="4" t="n"/>
-      <c r="D254" s="4" t="n"/>
+      <c r="C254" s="5" t="n">
+        <v>28.9496</v>
+      </c>
+      <c r="D254" s="5" t="n">
+        <v>32.4574</v>
+      </c>
       <c r="E254" s="5" t="n">
         <v>15.2721</v>
       </c>
@@ -20521,8 +21606,12 @@
       <c r="B255" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C255" s="4" t="n"/>
-      <c r="D255" s="4" t="n"/>
+      <c r="C255" s="5" t="n">
+        <v>28.3431</v>
+      </c>
+      <c r="D255" s="5" t="n">
+        <v>32.4945</v>
+      </c>
       <c r="E255" s="5" t="n">
         <v>16.2393</v>
       </c>
@@ -20578,8 +21667,12 @@
       <c r="B256" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C256" s="4" t="n"/>
-      <c r="D256" s="4" t="n"/>
+      <c r="C256" s="5" t="n">
+        <v>28.0644</v>
+      </c>
+      <c r="D256" s="5" t="n">
+        <v>32.2442</v>
+      </c>
       <c r="E256" s="5" t="n">
         <v>17.2154</v>
       </c>
@@ -20637,8 +21730,12 @@
       <c r="B257" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C257" s="4" t="n"/>
-      <c r="D257" s="4" t="n"/>
+      <c r="C257" s="5" t="n">
+        <v>27.8722</v>
+      </c>
+      <c r="D257" s="5" t="n">
+        <v>32.0657</v>
+      </c>
       <c r="E257" s="5" t="n">
         <v>17.1452</v>
       </c>
@@ -20694,8 +21791,12 @@
       <c r="B258" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C258" s="4" t="n"/>
-      <c r="D258" s="4" t="n"/>
+      <c r="C258" s="5" t="n">
+        <v>27.6866</v>
+      </c>
+      <c r="D258" s="5" t="n">
+        <v>31.7702</v>
+      </c>
       <c r="E258" s="5" t="n">
         <v>17.7604</v>
       </c>
@@ -20751,8 +21852,12 @@
       <c r="B259" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C259" s="4" t="n"/>
-      <c r="D259" s="4" t="n"/>
+      <c r="C259" s="5" t="n">
+        <v>27.4994</v>
+      </c>
+      <c r="D259" s="5" t="n">
+        <v>31.5118</v>
+      </c>
       <c r="E259" s="5" t="n">
         <v>17.9382</v>
       </c>
@@ -20812,8 +21917,12 @@
       <c r="B260" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C260" s="4" t="n"/>
-      <c r="D260" s="4" t="n"/>
+      <c r="C260" s="5" t="n">
+        <v>27.234</v>
+      </c>
+      <c r="D260" s="5" t="n">
+        <v>31.3004</v>
+      </c>
       <c r="E260" s="5" t="n">
         <v>18.9162</v>
       </c>
@@ -20869,8 +21978,12 @@
       <c r="B261" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C261" s="4" t="n"/>
-      <c r="D261" s="4" t="n"/>
+      <c r="C261" s="5" t="n">
+        <v>26.9262</v>
+      </c>
+      <c r="D261" s="5" t="n">
+        <v>31.1018</v>
+      </c>
       <c r="E261" s="5" t="n">
         <v>17.1093</v>
       </c>
@@ -20926,8 +22039,12 @@
       <c r="B262" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C262" s="4" t="n"/>
-      <c r="D262" s="4" t="n"/>
+      <c r="C262" s="5" t="n">
+        <v>26.8158</v>
+      </c>
+      <c r="D262" s="5" t="n">
+        <v>30.5539</v>
+      </c>
       <c r="E262" s="5" t="n">
         <v>15.5817</v>
       </c>
@@ -20987,8 +22104,12 @@
       <c r="B263" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C263" s="4" t="n"/>
-      <c r="D263" s="4" t="n"/>
+      <c r="C263" s="5" t="n">
+        <v>26.6051</v>
+      </c>
+      <c r="D263" s="5" t="n">
+        <v>30.2983</v>
+      </c>
       <c r="E263" s="5" t="n">
         <v>14.4681</v>
       </c>
@@ -21044,8 +22165,12 @@
       <c r="B264" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C264" s="4" t="n"/>
-      <c r="D264" s="4" t="n"/>
+      <c r="C264" s="5" t="n">
+        <v>26.2461</v>
+      </c>
+      <c r="D264" s="5" t="n">
+        <v>30.075</v>
+      </c>
       <c r="E264" s="5" t="n">
         <v>14.5463</v>
       </c>
@@ -21101,8 +22226,12 @@
       <c r="B265" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C265" s="4" t="n"/>
-      <c r="D265" s="4" t="n"/>
+      <c r="C265" s="5" t="n">
+        <v>25.7619</v>
+      </c>
+      <c r="D265" s="5" t="n">
+        <v>30.8335</v>
+      </c>
       <c r="E265" s="5" t="n">
         <v>14.2496</v>
       </c>
@@ -21276,8 +22405,12 @@
       <c r="B268" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C268" s="4" t="n"/>
-      <c r="D268" s="4" t="n"/>
+      <c r="C268" s="5" t="n">
+        <v>40.1994</v>
+      </c>
+      <c r="D268" s="5" t="n">
+        <v>44.6712</v>
+      </c>
       <c r="E268" s="5" t="n">
         <v>13.234</v>
       </c>
@@ -21333,8 +22466,12 @@
       <c r="B269" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C269" s="4" t="n"/>
-      <c r="D269" s="4" t="n"/>
+      <c r="C269" s="5" t="n">
+        <v>40.5188</v>
+      </c>
+      <c r="D269" s="5" t="n">
+        <v>44.1733</v>
+      </c>
       <c r="E269" s="5" t="n">
         <v>16.6229</v>
       </c>
@@ -21390,8 +22527,12 @@
       <c r="B270" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C270" s="4" t="n"/>
-      <c r="D270" s="4" t="n"/>
+      <c r="C270" s="5" t="n">
+        <v>40.5737</v>
+      </c>
+      <c r="D270" s="5" t="n">
+        <v>43.7813</v>
+      </c>
       <c r="E270" s="5" t="n">
         <v>16.5682</v>
       </c>
@@ -21447,8 +22588,12 @@
       <c r="B271" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C271" s="4" t="n"/>
-      <c r="D271" s="4" t="n"/>
+      <c r="C271" s="5" t="n">
+        <v>40.6005</v>
+      </c>
+      <c r="D271" s="5" t="n">
+        <v>42.9821</v>
+      </c>
       <c r="E271" s="5" t="n">
         <v>16.5513</v>
       </c>
@@ -21504,8 +22649,12 @@
       <c r="B272" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C272" s="4" t="n"/>
-      <c r="D272" s="4" t="n"/>
+      <c r="C272" s="5" t="n">
+        <v>40.3949</v>
+      </c>
+      <c r="D272" s="5" t="n">
+        <v>42.7871</v>
+      </c>
       <c r="E272" s="5" t="n">
         <v>15.8181</v>
       </c>
@@ -21561,8 +22710,12 @@
       <c r="B273" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C273" s="4" t="n"/>
-      <c r="D273" s="4" t="n"/>
+      <c r="C273" s="5" t="n">
+        <v>39.9346</v>
+      </c>
+      <c r="D273" s="5" t="n">
+        <v>44.5583</v>
+      </c>
       <c r="E273" s="5" t="n">
         <v>12.9564</v>
       </c>
@@ -21618,8 +22771,12 @@
       <c r="B274" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C274" s="4" t="n"/>
-      <c r="D274" s="4" t="n"/>
+      <c r="C274" s="5" t="n">
+        <v>40.0773</v>
+      </c>
+      <c r="D274" s="5" t="n">
+        <v>43.5487</v>
+      </c>
       <c r="E274" s="5" t="n">
         <v>13.0483</v>
       </c>
@@ -21675,8 +22832,12 @@
       <c r="B275" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C275" s="4" t="n"/>
-      <c r="D275" s="4" t="n"/>
+      <c r="C275" s="5" t="n">
+        <v>40.1859</v>
+      </c>
+      <c r="D275" s="5" t="n">
+        <v>42.9716</v>
+      </c>
       <c r="E275" s="5" t="n">
         <v>13.9542</v>
       </c>
@@ -21734,8 +22895,12 @@
       <c r="B276" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C276" s="4" t="n"/>
-      <c r="D276" s="4" t="n"/>
+      <c r="C276" s="5" t="n">
+        <v>40.1975</v>
+      </c>
+      <c r="D276" s="5" t="n">
+        <v>42.5913</v>
+      </c>
       <c r="E276" s="5" t="n">
         <v>13.7547</v>
       </c>
@@ -21791,8 +22956,12 @@
       <c r="B277" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C277" s="4" t="n"/>
-      <c r="D277" s="4" t="n"/>
+      <c r="C277" s="5" t="n">
+        <v>40.007</v>
+      </c>
+      <c r="D277" s="5" t="n">
+        <v>42.6398</v>
+      </c>
       <c r="E277" s="5" t="n">
         <v>12.9335</v>
       </c>
@@ -21848,8 +23017,12 @@
       <c r="B278" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C278" s="4" t="n"/>
-      <c r="D278" s="4" t="n"/>
+      <c r="C278" s="5" t="n">
+        <v>39.7733</v>
+      </c>
+      <c r="D278" s="5" t="n">
+        <v>42.5182</v>
+      </c>
       <c r="E278" s="5" t="n">
         <v>13.2554</v>
       </c>
@@ -21909,8 +23082,12 @@
       <c r="B279" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C279" s="4" t="n"/>
-      <c r="D279" s="4" t="n"/>
+      <c r="C279" s="5" t="n">
+        <v>39.7398</v>
+      </c>
+      <c r="D279" s="5" t="n">
+        <v>42.72</v>
+      </c>
       <c r="E279" s="5" t="n">
         <v>10.6421</v>
       </c>
@@ -21966,8 +23143,12 @@
       <c r="B280" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C280" s="4" t="n"/>
-      <c r="D280" s="4" t="n"/>
+      <c r="C280" s="5" t="n">
+        <v>39.7079</v>
+      </c>
+      <c r="D280" s="5" t="n">
+        <v>42.8059</v>
+      </c>
       <c r="E280" s="5" t="n">
         <v>9.1831</v>
       </c>
@@ -22023,8 +23204,12 @@
       <c r="B281" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C281" s="4" t="n"/>
-      <c r="D281" s="4" t="n"/>
+      <c r="C281" s="5" t="n">
+        <v>39.7174</v>
+      </c>
+      <c r="D281" s="5" t="n">
+        <v>42.5112</v>
+      </c>
       <c r="E281" s="5" t="n">
         <v>10.2884</v>
       </c>
@@ -22084,8 +23269,12 @@
       <c r="B282" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C282" s="4" t="n"/>
-      <c r="D282" s="4" t="n"/>
+      <c r="C282" s="5" t="n">
+        <v>39.7487</v>
+      </c>
+      <c r="D282" s="5" t="n">
+        <v>41.9168</v>
+      </c>
       <c r="E282" s="5" t="n">
         <v>11.4688</v>
       </c>
@@ -22141,8 +23330,12 @@
       <c r="B283" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C283" s="4" t="n"/>
-      <c r="D283" s="4" t="n"/>
+      <c r="C283" s="5" t="n">
+        <v>39.5939</v>
+      </c>
+      <c r="D283" s="5" t="n">
+        <v>41.7804</v>
+      </c>
       <c r="E283" s="5" t="n">
         <v>10.9384</v>
       </c>
@@ -22198,8 +23391,12 @@
       <c r="B284" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C284" s="4" t="n"/>
-      <c r="D284" s="4" t="n"/>
+      <c r="C284" s="5" t="n">
+        <v>39.0937</v>
+      </c>
+      <c r="D284" s="5" t="n">
+        <v>43.0736</v>
+      </c>
       <c r="E284" s="5" t="n">
         <v>10.7991</v>
       </c>
@@ -23454,8 +24651,12 @@
       <c r="B306" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C306" s="4" t="n"/>
-      <c r="D306" s="4" t="n"/>
+      <c r="C306" s="5" t="n">
+        <v>40.0794</v>
+      </c>
+      <c r="D306" s="5" t="n">
+        <v>42.206</v>
+      </c>
       <c r="E306" s="5" t="n">
         <v>9.821</v>
       </c>
@@ -23507,8 +24708,12 @@
       <c r="B307" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C307" s="4" t="n"/>
-      <c r="D307" s="4" t="n"/>
+      <c r="C307" s="5" t="n">
+        <v>40.4902</v>
+      </c>
+      <c r="D307" s="5" t="n">
+        <v>42.2759</v>
+      </c>
       <c r="E307" s="5" t="n"/>
       <c r="F307" s="5" t="n"/>
       <c r="G307" s="5" t="n"/>
@@ -23560,8 +24765,12 @@
       <c r="B308" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C308" s="4" t="n"/>
-      <c r="D308" s="4" t="n"/>
+      <c r="C308" s="5" t="n">
+        <v>40.778</v>
+      </c>
+      <c r="D308" s="5" t="n">
+        <v>41.7016</v>
+      </c>
       <c r="E308" s="5" t="n"/>
       <c r="F308" s="5" t="n"/>
       <c r="G308" s="5" t="n"/>
@@ -23613,8 +24822,12 @@
       <c r="B309" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C309" s="4" t="n"/>
-      <c r="D309" s="4" t="n"/>
+      <c r="C309" s="5" t="n">
+        <v>41.0031</v>
+      </c>
+      <c r="D309" s="5" t="n">
+        <v>41.2537</v>
+      </c>
       <c r="E309" s="5" t="n"/>
       <c r="F309" s="5" t="n"/>
       <c r="G309" s="5" t="n"/>
@@ -23668,8 +24881,12 @@
       <c r="B310" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C310" s="4" t="n"/>
-      <c r="D310" s="4" t="n"/>
+      <c r="C310" s="5" t="n">
+        <v>41.1581</v>
+      </c>
+      <c r="D310" s="5" t="n">
+        <v>40.857</v>
+      </c>
       <c r="E310" s="5" t="n"/>
       <c r="F310" s="5" t="n"/>
       <c r="G310" s="5" t="n"/>
@@ -23723,8 +24940,12 @@
       <c r="B311" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C311" s="4" t="n"/>
-      <c r="D311" s="4" t="n"/>
+      <c r="C311" s="5" t="n">
+        <v>41.3139</v>
+      </c>
+      <c r="D311" s="5" t="n">
+        <v>41.1989</v>
+      </c>
       <c r="E311" s="5" t="n"/>
       <c r="F311" s="5" t="n"/>
       <c r="G311" s="5" t="n"/>
@@ -23778,8 +24999,12 @@
       <c r="B312" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C312" s="4" t="n"/>
-      <c r="D312" s="4" t="n"/>
+      <c r="C312" s="5" t="n">
+        <v>41.539</v>
+      </c>
+      <c r="D312" s="5" t="n">
+        <v>40.8445</v>
+      </c>
       <c r="E312" s="5" t="n"/>
       <c r="F312" s="5" t="n"/>
       <c r="G312" s="5" t="n"/>
@@ -23833,8 +25058,12 @@
       <c r="B313" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C313" s="4" t="n"/>
-      <c r="D313" s="4" t="n"/>
+      <c r="C313" s="5" t="n">
+        <v>41.475</v>
+      </c>
+      <c r="D313" s="5" t="n">
+        <v>40.7656</v>
+      </c>
       <c r="E313" s="5" t="n"/>
       <c r="F313" s="5" t="n">
         <v>2.5349</v>
@@ -23890,8 +25119,12 @@
       <c r="B314" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C314" s="4" t="n"/>
-      <c r="D314" s="4" t="n"/>
+      <c r="C314" s="5" t="n">
+        <v>42.0564</v>
+      </c>
+      <c r="D314" s="5" t="n">
+        <v>40.295</v>
+      </c>
       <c r="E314" s="5" t="n"/>
       <c r="F314" s="5" t="n"/>
       <c r="G314" s="5" t="n"/>
@@ -23945,8 +25178,12 @@
       <c r="B315" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C315" s="4" t="n"/>
-      <c r="D315" s="4" t="n"/>
+      <c r="C315" s="5" t="n">
+        <v>42.4303</v>
+      </c>
+      <c r="D315" s="5" t="n">
+        <v>40.2008</v>
+      </c>
       <c r="E315" s="5" t="n"/>
       <c r="F315" s="5" t="n"/>
       <c r="G315" s="5" t="n"/>
@@ -24000,8 +25237,12 @@
       <c r="B316" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C316" s="4" t="n"/>
-      <c r="D316" s="4" t="n"/>
+      <c r="C316" s="5" t="n">
+        <v>42.2822</v>
+      </c>
+      <c r="D316" s="5" t="n">
+        <v>39.7462</v>
+      </c>
       <c r="E316" s="5" t="n"/>
       <c r="F316" s="5" t="n">
         <v>11.4592</v>
@@ -24059,8 +25300,12 @@
       <c r="B317" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C317" s="4" t="n"/>
-      <c r="D317" s="4" t="n"/>
+      <c r="C317" s="5" t="n">
+        <v>43.011</v>
+      </c>
+      <c r="D317" s="5" t="n">
+        <v>39.4062</v>
+      </c>
       <c r="E317" s="5" t="n"/>
       <c r="F317" s="5" t="n"/>
       <c r="G317" s="5" t="n"/>
@@ -24114,8 +25359,12 @@
       <c r="B318" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C318" s="4" t="n"/>
-      <c r="D318" s="4" t="n"/>
+      <c r="C318" s="5" t="n">
+        <v>43.2744</v>
+      </c>
+      <c r="D318" s="5" t="n">
+        <v>38.8824</v>
+      </c>
       <c r="E318" s="5" t="n"/>
       <c r="F318" s="5" t="n"/>
       <c r="G318" s="5" t="n"/>
@@ -24169,8 +25418,12 @@
       <c r="B319" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C319" s="4" t="n"/>
-      <c r="D319" s="4" t="n"/>
+      <c r="C319" s="5" t="n">
+        <v>43.0029</v>
+      </c>
+      <c r="D319" s="5" t="n">
+        <v>38.6427</v>
+      </c>
       <c r="E319" s="5" t="n"/>
       <c r="F319" s="5" t="n">
         <v>47.0244</v>
@@ -24226,8 +25479,12 @@
       <c r="B320" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C320" s="4" t="n"/>
-      <c r="D320" s="4" t="n"/>
+      <c r="C320" s="5" t="n">
+        <v>42.9983</v>
+      </c>
+      <c r="D320" s="5" t="n">
+        <v>38.485</v>
+      </c>
       <c r="E320" s="5" t="n"/>
       <c r="F320" s="5" t="n"/>
       <c r="G320" s="5" t="n"/>
@@ -24277,8 +25534,12 @@
       <c r="B321" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C321" s="4" t="n"/>
-      <c r="D321" s="4" t="n"/>
+      <c r="C321" s="5" t="n">
+        <v>43.2154</v>
+      </c>
+      <c r="D321" s="5" t="n">
+        <v>37.5825</v>
+      </c>
       <c r="E321" s="5" t="n"/>
       <c r="F321" s="5" t="n"/>
       <c r="G321" s="5" t="n"/>
@@ -24330,8 +25591,12 @@
       <c r="B322" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C322" s="4" t="n"/>
-      <c r="D322" s="4" t="n"/>
+      <c r="C322" s="5" t="n">
+        <v>43.002</v>
+      </c>
+      <c r="D322" s="5" t="n">
+        <v>37.6737</v>
+      </c>
       <c r="E322" s="5" t="n"/>
       <c r="F322" s="5" t="n"/>
       <c r="G322" s="5" t="n"/>
@@ -25422,8 +26687,12 @@
       <c r="B344" s="3" t="n">
         <v>2004</v>
       </c>
-      <c r="C344" s="4" t="n"/>
-      <c r="D344" s="4" t="n"/>
+      <c r="C344" s="5" t="n">
+        <v>46.2416</v>
+      </c>
+      <c r="D344" s="5" t="n">
+        <v>48.7402</v>
+      </c>
       <c r="E344" s="5" t="n">
         <v>12.8141</v>
       </c>
@@ -25477,8 +26746,12 @@
       <c r="B345" s="3" t="n">
         <v>2005</v>
       </c>
-      <c r="C345" s="4" t="n"/>
-      <c r="D345" s="4" t="n"/>
+      <c r="C345" s="5" t="n">
+        <v>46.6956</v>
+      </c>
+      <c r="D345" s="5" t="n">
+        <v>48.4587</v>
+      </c>
       <c r="E345" s="5" t="n">
         <v>16.5288</v>
       </c>
@@ -25534,8 +26807,12 @@
       <c r="B346" s="3" t="n">
         <v>2006</v>
       </c>
-      <c r="C346" s="4" t="n"/>
-      <c r="D346" s="4" t="n"/>
+      <c r="C346" s="5" t="n">
+        <v>46.8109</v>
+      </c>
+      <c r="D346" s="5" t="n">
+        <v>47.6212</v>
+      </c>
       <c r="E346" s="5" t="n">
         <v>17.0922</v>
       </c>
@@ -25591,8 +26868,12 @@
       <c r="B347" s="3" t="n">
         <v>2007</v>
       </c>
-      <c r="C347" s="4" t="n"/>
-      <c r="D347" s="4" t="n"/>
+      <c r="C347" s="5" t="n">
+        <v>46.8001</v>
+      </c>
+      <c r="D347" s="5" t="n">
+        <v>46.7381</v>
+      </c>
       <c r="E347" s="5" t="n">
         <v>15.818</v>
       </c>
@@ -25648,8 +26929,12 @@
       <c r="B348" s="3" t="n">
         <v>2008</v>
       </c>
-      <c r="C348" s="4" t="n"/>
-      <c r="D348" s="4" t="n"/>
+      <c r="C348" s="5" t="n">
+        <v>46.754</v>
+      </c>
+      <c r="D348" s="5" t="n">
+        <v>46.473</v>
+      </c>
       <c r="E348" s="5" t="n">
         <v>17.0917</v>
       </c>
@@ -25705,8 +26990,12 @@
       <c r="B349" s="3" t="n">
         <v>2009</v>
       </c>
-      <c r="C349" s="4" t="n"/>
-      <c r="D349" s="4" t="n"/>
+      <c r="C349" s="5" t="n">
+        <v>46.3122</v>
+      </c>
+      <c r="D349" s="5" t="n">
+        <v>49.2124</v>
+      </c>
       <c r="E349" s="5" t="n">
         <v>15.7892</v>
       </c>
@@ -25762,8 +27051,12 @@
       <c r="B350" s="3" t="n">
         <v>2010</v>
       </c>
-      <c r="C350" s="4" t="n"/>
-      <c r="D350" s="4" t="n"/>
+      <c r="C350" s="5" t="n">
+        <v>46.3568</v>
+      </c>
+      <c r="D350" s="5" t="n">
+        <v>48.6768</v>
+      </c>
       <c r="E350" s="5" t="n">
         <v>14.9975</v>
       </c>
@@ -25819,8 +27112,12 @@
       <c r="B351" s="3" t="n">
         <v>2011</v>
       </c>
-      <c r="C351" s="4" t="n"/>
-      <c r="D351" s="4" t="n"/>
+      <c r="C351" s="5" t="n">
+        <v>46.4594</v>
+      </c>
+      <c r="D351" s="5" t="n">
+        <v>47.4782</v>
+      </c>
       <c r="E351" s="5" t="n">
         <v>17.84</v>
       </c>
@@ -25878,8 +27175,12 @@
       <c r="B352" s="3" t="n">
         <v>2012</v>
       </c>
-      <c r="C352" s="4" t="n"/>
-      <c r="D352" s="4" t="n"/>
+      <c r="C352" s="5" t="n">
+        <v>46.5442</v>
+      </c>
+      <c r="D352" s="5" t="n">
+        <v>47.6002</v>
+      </c>
       <c r="E352" s="5" t="n">
         <v>17.6333</v>
       </c>
@@ -25935,8 +27236,12 @@
       <c r="B353" s="3" t="n">
         <v>2013</v>
       </c>
-      <c r="C353" s="4" t="n"/>
-      <c r="D353" s="4" t="n"/>
+      <c r="C353" s="5" t="n">
+        <v>46.715</v>
+      </c>
+      <c r="D353" s="5" t="n">
+        <v>47.5637</v>
+      </c>
       <c r="E353" s="5" t="n">
         <v>16.8987</v>
       </c>
@@ -25992,8 +27297,12 @@
       <c r="B354" s="3" t="n">
         <v>2014</v>
       </c>
-      <c r="C354" s="4" t="n"/>
-      <c r="D354" s="4" t="n"/>
+      <c r="C354" s="5" t="n">
+        <v>45.9817</v>
+      </c>
+      <c r="D354" s="5" t="n">
+        <v>47.5931</v>
+      </c>
       <c r="E354" s="5" t="n">
         <v>17.2943</v>
       </c>
@@ -26053,8 +27362,12 @@
       <c r="B355" s="3" t="n">
         <v>2015</v>
       </c>
-      <c r="C355" s="4" t="n"/>
-      <c r="D355" s="4" t="n"/>
+      <c r="C355" s="5" t="n">
+        <v>45.0853</v>
+      </c>
+      <c r="D355" s="5" t="n">
+        <v>47.7882</v>
+      </c>
       <c r="E355" s="5" t="n">
         <v>20.4514</v>
       </c>
@@ -26110,8 +27423,12 @@
       <c r="B356" s="3" t="n">
         <v>2016</v>
       </c>
-      <c r="C356" s="4" t="n"/>
-      <c r="D356" s="4" t="n"/>
+      <c r="C356" s="5" t="n">
+        <v>45.2024</v>
+      </c>
+      <c r="D356" s="5" t="n">
+        <v>47.5206</v>
+      </c>
       <c r="E356" s="5" t="n">
         <v>19.6301</v>
       </c>
@@ -26167,8 +27484,12 @@
       <c r="B357" s="3" t="n">
         <v>2017</v>
       </c>
-      <c r="C357" s="4" t="n"/>
-      <c r="D357" s="4" t="n"/>
+      <c r="C357" s="5" t="n">
+        <v>45.2354</v>
+      </c>
+      <c r="D357" s="5" t="n">
+        <v>47.8649</v>
+      </c>
       <c r="E357" s="5" t="n">
         <v>20.0524</v>
       </c>
@@ -26228,8 +27549,12 @@
       <c r="B358" s="3" t="n">
         <v>2018</v>
       </c>
-      <c r="C358" s="4" t="n"/>
-      <c r="D358" s="4" t="n"/>
+      <c r="C358" s="5" t="n">
+        <v>45.5438</v>
+      </c>
+      <c r="D358" s="5" t="n">
+        <v>47.3939</v>
+      </c>
       <c r="E358" s="5" t="n">
         <v>20.1426</v>
       </c>
@@ -26285,8 +27610,12 @@
       <c r="B359" s="3" t="n">
         <v>2019</v>
       </c>
-      <c r="C359" s="4" t="n"/>
-      <c r="D359" s="4" t="n"/>
+      <c r="C359" s="5" t="n">
+        <v>45.9374</v>
+      </c>
+      <c r="D359" s="5" t="n">
+        <v>46.5629</v>
+      </c>
       <c r="E359" s="5" t="n">
         <v>19.1961</v>
       </c>
@@ -26342,8 +27671,12 @@
       <c r="B360" s="3" t="n">
         <v>2020</v>
       </c>
-      <c r="C360" s="4" t="n"/>
-      <c r="D360" s="4" t="n"/>
+      <c r="C360" s="5" t="n">
+        <v>46.0136</v>
+      </c>
+      <c r="D360" s="5" t="n">
+        <v>46.9246</v>
+      </c>
       <c r="E360" s="5" t="n">
         <v>19.1514</v>
       </c>

</xml_diff>

<commit_message>
Document sourcing investigation for remaining blank columns in READ_ME
</commit_message>
<xml_diff>
--- a/DFS_data_FILLED.xlsx
+++ b/DFS_data_FILLED.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -606,6 +606,79 @@
       <c r="A22" t="inlineStr">
         <is>
           <t xml:space="preserve">  - This means the paper's main dependent variable is missing for 2 of the 5 core countries - a real feasibility issue to resolve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>SOURCING INVESTIGATION - remaining blank columns (checked, genuinely not auto-fetchable):</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - CASH (currency/M2): IMF IFS is NOT yet on the new IMF SDMX API (api.imf.org); WDI has broad money but</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    not currency in circulation. Must be taken from IMF IFS legacy tables or national central banks manually.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - POS terminals: NOT a separate indicator in the current IMF FAS codelist (only ATMs, cards, mobile money).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - CASHLESS_VAL (value of card/e-payments % GDP): not available for these countries via FAS/BIS open data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - MOBILE_COVERAGE (3G/4G): ITU only; no open API / not in WDI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - UZB &amp; TKM SHADOW: not in WB DGE/MIMIC; only in Medina &amp; Schneider (2018) / Asllani-Schneider (2024), PDF only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>RECOMMENDATION: DFS_INDEX can still be built from 3 real components (ACCOUNT, DIGPAY, ATM_per100k).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>POS and CASHLESS_VAL can be dropped from the composite with a footnote. CASH channel (H3) needs the manual IFS series.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Everything green in this file is REAL and verifiable. Nothing was fabricated.</t>
         </is>
       </c>
     </row>

</xml_diff>